<commit_message>
Changed starting year to 1994
</commit_message>
<xml_diff>
--- a/FinalDataset.xlsx
+++ b/FinalDataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rneribar/AIMM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/krishnaprasadpa/Desktop/Part time/aimm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93EC8C38-1433-D74E-8DE7-054D9F9F4E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EBD4DBD-4DAB-2842-8A66-5DCAE2477367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1180" yWindow="760" windowWidth="29060" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.Original" sheetId="28" r:id="rId1"/>
@@ -7568,7 +7568,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36E17C31-AD61-3D47-86B4-5BD830528393}">
-  <dimension ref="A1:AF37"/>
+  <dimension ref="A1:AF36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="5"/>
@@ -7974,3263 +7974,3165 @@
         <v>46</v>
       </c>
       <c r="B5" s="9">
-        <f>MAX(B6:B37)</f>
+        <f>MAX(B6:B36)</f>
         <v>3.4064709999999998</v>
       </c>
       <c r="C5" s="9">
-        <f t="shared" ref="C5:AF5" si="0">MAX(C6:C37)</f>
-        <v>161027.252457</v>
+        <f>MAX(C6:C36)</f>
+        <v>154688.542193</v>
       </c>
       <c r="D5" s="9">
-        <f t="shared" si="0"/>
-        <v>1.7171270000000001</v>
+        <f>MAX(D6:D36)</f>
+        <v>1.583216</v>
       </c>
       <c r="E5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(E6:E36)</f>
         <v>28180.264358</v>
       </c>
       <c r="F5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(F6:F36)</f>
         <v>17.510000000000002</v>
       </c>
       <c r="G5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(G6:G36)</f>
         <v>72.8</v>
       </c>
       <c r="H5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(H6:H36)</f>
         <v>15.456422</v>
       </c>
       <c r="I5" s="9">
-        <f t="shared" si="0"/>
-        <v>635.51794600000005</v>
+        <f>MAX(I6:I36)</f>
+        <v>611.711996</v>
       </c>
       <c r="J5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(J6:J36)</f>
         <v>667.17</v>
       </c>
       <c r="K5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(K6:K36)</f>
         <v>16.311599999999999</v>
       </c>
       <c r="L5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(L6:L36)</f>
         <v>46.861249999999998</v>
       </c>
       <c r="M5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(M6:M36)</f>
         <v>90880</v>
       </c>
       <c r="N5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(N6:N36)</f>
         <v>125650</v>
       </c>
       <c r="O5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(O6:O36)</f>
         <v>393586.7</v>
       </c>
       <c r="P5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(P6:P36)</f>
         <v>91721</v>
       </c>
       <c r="Q5" s="19">
-        <f t="shared" si="0"/>
-        <v>21321</v>
+        <f>MAX(Q6:Q36)</f>
+        <v>14923</v>
       </c>
       <c r="R5" s="19">
-        <f t="shared" si="0"/>
+        <f>MAX(R6:R36)</f>
         <v>40932</v>
       </c>
       <c r="S5" s="19">
-        <f t="shared" si="0"/>
+        <f>MAX(S6:S36)</f>
         <v>98742</v>
       </c>
       <c r="T5" s="19">
-        <f t="shared" si="0"/>
+        <f>MAX(T6:T36)</f>
         <v>25761</v>
       </c>
       <c r="U5" s="19">
-        <f t="shared" si="0"/>
+        <f>MAX(U6:U36)</f>
         <v>76683</v>
       </c>
       <c r="V5" s="19">
-        <f t="shared" si="0"/>
+        <f>MAX(V6:V36)</f>
         <v>91181</v>
       </c>
       <c r="W5" s="19">
-        <f t="shared" si="0"/>
+        <f>MAX(W6:W36)</f>
         <v>277830</v>
       </c>
       <c r="X5" s="19">
-        <f t="shared" si="0"/>
+        <f>MAX(X6:X36)</f>
         <v>69313</v>
       </c>
       <c r="Y5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(Y6:Y36)</f>
         <v>96.26</v>
       </c>
       <c r="Z5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(Z6:Z36)</f>
         <v>299.56</v>
       </c>
       <c r="AA5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(AA6:AA36)</f>
         <v>2116.8000000000002</v>
       </c>
       <c r="AB5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(AB6:AB36)</f>
         <v>374960</v>
       </c>
       <c r="AC5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(AC6:AC36)</f>
         <v>497040</v>
       </c>
       <c r="AD5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(AD6:AD36)</f>
         <v>60000</v>
       </c>
       <c r="AE5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(AE6:AE36)</f>
         <v>3320.7</v>
       </c>
       <c r="AF5" s="9">
-        <f t="shared" si="0"/>
+        <f>MAX(AF6:AF36)</f>
         <v>2183.1999999999998</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" s="10">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="B6" s="11">
-        <v>0.86631400000000003</v>
+        <v>1.0651360000000001</v>
       </c>
       <c r="C6" s="11">
-        <v>161027.252457</v>
+        <v>154688.542193</v>
       </c>
       <c r="D6" s="11">
-        <v>1.7171270000000001</v>
+        <v>1.531957</v>
       </c>
       <c r="E6" s="11">
-        <v>20542.634612000002</v>
+        <v>17835.29912</v>
       </c>
       <c r="F6" s="11">
-        <v>6.3890000000000002</v>
+        <v>5.48</v>
       </c>
       <c r="G6" s="11">
-        <v>67.959999999999994</v>
+        <v>67.400000000000006</v>
       </c>
       <c r="H6" s="11">
-        <v>15.164866</v>
+        <v>14.255712000000001</v>
       </c>
       <c r="I6" s="11">
-        <v>635.51794600000005</v>
+        <v>611.711996</v>
       </c>
       <c r="J6" s="11">
-        <v>149.47</v>
+        <v>136.85</v>
       </c>
       <c r="K6" s="11">
-        <v>10.553838000000001</v>
+        <v>10.957749</v>
       </c>
       <c r="L6" s="11">
-        <v>12.317608999999999</v>
+        <v>18.130517000000001</v>
       </c>
       <c r="M6" s="11">
-        <v>89017</v>
+        <v>42745</v>
       </c>
       <c r="N6" s="11">
-        <v>90817</v>
+        <v>118638</v>
       </c>
       <c r="O6" s="11">
-        <v>199380</v>
+        <v>180691</v>
       </c>
       <c r="P6" s="11">
-        <v>56591</v>
+        <v>41233</v>
       </c>
       <c r="Q6" s="20">
-        <v>21321</v>
+        <v>5250</v>
       </c>
       <c r="R6" s="20">
-        <v>16169</v>
+        <v>33406</v>
       </c>
       <c r="S6" s="20">
-        <v>50480</v>
+        <v>43846</v>
       </c>
       <c r="T6" s="20">
-        <v>10968</v>
+        <v>6442</v>
       </c>
       <c r="U6" s="20">
-        <v>67581</v>
+        <v>37450</v>
       </c>
       <c r="V6" s="20">
-        <v>74599</v>
+        <v>85209</v>
       </c>
       <c r="W6" s="20">
-        <v>148731</v>
+        <v>136786</v>
       </c>
       <c r="X6" s="20">
-        <v>45615</v>
+        <v>34790</v>
       </c>
       <c r="Y6" s="11">
-        <v>40.51</v>
+        <v>51.76</v>
       </c>
       <c r="Z6" s="11">
-        <v>273.62</v>
+        <v>274.06</v>
       </c>
       <c r="AA6" s="11">
-        <v>529</v>
+        <v>550</v>
       </c>
       <c r="AB6" s="11">
-        <v>371274.9</v>
+        <v>354363</v>
       </c>
       <c r="AC6" s="11">
-        <v>492155.1</v>
+        <v>469737</v>
       </c>
       <c r="AD6" s="11">
         <v>60000</v>
       </c>
       <c r="AE6" s="11">
-        <v>1168.9000000000001</v>
+        <v>1073.5</v>
       </c>
       <c r="AF6" s="11">
-        <v>681.24324300000001</v>
+        <v>686.27026999999998</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" s="10">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="B7" s="11">
-        <v>1.0651360000000001</v>
+        <v>1.2508440000000001</v>
       </c>
       <c r="C7" s="11">
-        <v>154688.542193</v>
+        <v>117744.159965</v>
       </c>
       <c r="D7" s="11">
-        <v>1.531957</v>
+        <v>1.583216</v>
       </c>
       <c r="E7" s="11">
-        <v>17835.29912</v>
+        <v>28180.264358</v>
       </c>
       <c r="F7" s="11">
-        <v>5.48</v>
+        <v>8.06</v>
       </c>
       <c r="G7" s="11">
-        <v>67.400000000000006</v>
+        <v>65.900000000000006</v>
       </c>
       <c r="H7" s="11">
-        <v>14.255712000000001</v>
+        <v>15.087118</v>
       </c>
       <c r="I7" s="11">
-        <v>611.711996</v>
+        <v>466.48844400000002</v>
       </c>
       <c r="J7" s="11">
-        <v>136.85</v>
+        <v>157.05000000000001</v>
       </c>
       <c r="K7" s="11">
-        <v>10.957749</v>
+        <v>10.865208000000001</v>
       </c>
       <c r="L7" s="11">
-        <v>18.130517000000001</v>
+        <v>14.371081</v>
       </c>
       <c r="M7" s="11">
-        <v>42745</v>
+        <v>72882</v>
       </c>
       <c r="N7" s="11">
-        <v>118638</v>
+        <v>119193</v>
       </c>
       <c r="O7" s="11">
-        <v>180691</v>
+        <v>218155</v>
       </c>
       <c r="P7" s="11">
-        <v>41233</v>
+        <v>72977</v>
       </c>
       <c r="Q7" s="20">
-        <v>5250</v>
+        <v>8698</v>
       </c>
       <c r="R7" s="20">
-        <v>33406</v>
+        <v>27955</v>
       </c>
       <c r="S7" s="20">
-        <v>43846</v>
+        <v>54055</v>
       </c>
       <c r="T7" s="20">
-        <v>6442</v>
+        <v>19492</v>
       </c>
       <c r="U7" s="20">
-        <v>37450</v>
+        <v>64019</v>
       </c>
       <c r="V7" s="20">
-        <v>85209</v>
+        <v>91181</v>
       </c>
       <c r="W7" s="20">
-        <v>136786</v>
+        <v>163967</v>
       </c>
       <c r="X7" s="20">
-        <v>34790</v>
+        <v>53484</v>
       </c>
       <c r="Y7" s="11">
-        <v>51.76</v>
+        <v>62.27</v>
       </c>
       <c r="Z7" s="11">
-        <v>274.06</v>
+        <v>277.35000000000002</v>
       </c>
       <c r="AA7" s="11">
-        <v>550</v>
+        <v>622</v>
       </c>
       <c r="AB7" s="11">
-        <v>354363</v>
+        <v>374960</v>
       </c>
       <c r="AC7" s="11">
-        <v>469737</v>
+        <v>497040</v>
       </c>
       <c r="AD7" s="11">
         <v>60000</v>
       </c>
       <c r="AE7" s="11">
-        <v>1073.5</v>
+        <v>1140</v>
       </c>
       <c r="AF7" s="11">
-        <v>686.27026999999998</v>
+        <v>691.29729699999996</v>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" s="10">
-        <v>1995</v>
+        <v>1996</v>
       </c>
       <c r="B8" s="11">
-        <v>1.2508440000000001</v>
+        <v>1.2888280000000001</v>
       </c>
       <c r="C8" s="11">
-        <v>117744.159965</v>
+        <v>89958.493008000005</v>
       </c>
       <c r="D8" s="11">
-        <v>1.583216</v>
+        <v>1.4175089999999999</v>
       </c>
       <c r="E8" s="11">
-        <v>28180.264358</v>
+        <v>21739.013164</v>
       </c>
       <c r="F8" s="11">
-        <v>8.06</v>
+        <v>8.23</v>
       </c>
       <c r="G8" s="11">
-        <v>65.900000000000006</v>
+        <v>66.599999999999994</v>
       </c>
       <c r="H8" s="11">
-        <v>15.087118</v>
+        <v>14.275625</v>
       </c>
       <c r="I8" s="11">
-        <v>466.48844400000002</v>
+        <v>357.03637700000002</v>
       </c>
       <c r="J8" s="11">
-        <v>157.05000000000001</v>
+        <v>160.80000000000001</v>
       </c>
       <c r="K8" s="11">
-        <v>10.865208000000001</v>
+        <v>10.535812999999999</v>
       </c>
       <c r="L8" s="11">
-        <v>14.371081</v>
+        <v>13.186002999999999</v>
       </c>
       <c r="M8" s="11">
-        <v>72882</v>
+        <v>59260</v>
       </c>
       <c r="N8" s="11">
-        <v>119193</v>
+        <v>125156</v>
       </c>
       <c r="O8" s="11">
-        <v>218155</v>
+        <v>183400</v>
       </c>
       <c r="P8" s="11">
-        <v>72977</v>
+        <v>75141</v>
       </c>
       <c r="Q8" s="20">
-        <v>8698</v>
+        <v>10383</v>
       </c>
       <c r="R8" s="20">
-        <v>27955</v>
+        <v>40932</v>
       </c>
       <c r="S8" s="20">
-        <v>54055</v>
+        <v>54292</v>
       </c>
       <c r="T8" s="20">
-        <v>19492</v>
+        <v>21049</v>
       </c>
       <c r="U8" s="20">
-        <v>64019</v>
+        <v>48862</v>
       </c>
       <c r="V8" s="20">
-        <v>91181</v>
+        <v>84112</v>
       </c>
       <c r="W8" s="20">
-        <v>163967</v>
+        <v>129033</v>
       </c>
       <c r="X8" s="20">
-        <v>53484</v>
+        <v>54088</v>
       </c>
       <c r="Y8" s="11">
-        <v>62.27</v>
+        <v>65.75</v>
       </c>
       <c r="Z8" s="11">
-        <v>277.35000000000002</v>
+        <v>278.67</v>
       </c>
       <c r="AA8" s="11">
-        <v>622</v>
+        <v>659</v>
       </c>
       <c r="AB8" s="11">
-        <v>374960</v>
+        <v>305601</v>
       </c>
       <c r="AC8" s="11">
-        <v>497040</v>
+        <v>405099</v>
       </c>
       <c r="AD8" s="11">
         <v>60000</v>
       </c>
       <c r="AE8" s="11">
-        <v>1140</v>
+        <v>732</v>
       </c>
       <c r="AF8" s="11">
-        <v>691.29729699999996</v>
+        <v>652</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" s="10">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="B9" s="11">
-        <v>1.2888280000000001</v>
+        <v>1.520661</v>
       </c>
       <c r="C9" s="11">
-        <v>89958.493008000005</v>
+        <v>76542.059815000001</v>
       </c>
       <c r="D9" s="11">
-        <v>1.4175089999999999</v>
+        <v>1.3006169999999999</v>
       </c>
       <c r="E9" s="11">
-        <v>21739.013164</v>
+        <v>18161.02189</v>
       </c>
       <c r="F9" s="11">
-        <v>8.23</v>
+        <v>9.6300000000000008</v>
       </c>
       <c r="G9" s="11">
-        <v>66.599999999999994</v>
+        <v>63.9</v>
       </c>
       <c r="H9" s="11">
-        <v>14.275625</v>
+        <v>13.968859999999999</v>
       </c>
       <c r="I9" s="11">
-        <v>357.03637700000002</v>
+        <v>304.29779300000001</v>
       </c>
       <c r="J9" s="11">
-        <v>160.80000000000001</v>
+        <v>160.55000000000001</v>
       </c>
       <c r="K9" s="11">
-        <v>10.535812999999999</v>
+        <v>10.903962</v>
       </c>
       <c r="L9" s="11">
-        <v>13.186002999999999</v>
+        <v>14.352134</v>
       </c>
       <c r="M9" s="11">
-        <v>59260</v>
+        <v>44298</v>
       </c>
       <c r="N9" s="11">
-        <v>125156</v>
+        <v>114972</v>
       </c>
       <c r="O9" s="11">
-        <v>183400</v>
+        <v>198846</v>
       </c>
       <c r="P9" s="11">
-        <v>75141</v>
+        <v>88247</v>
       </c>
       <c r="Q9" s="20">
-        <v>10383</v>
+        <v>3585</v>
       </c>
       <c r="R9" s="20">
-        <v>40932</v>
+        <v>35860</v>
       </c>
       <c r="S9" s="20">
-        <v>54292</v>
+        <v>46382</v>
       </c>
       <c r="T9" s="20">
-        <v>21049</v>
+        <v>18934</v>
       </c>
       <c r="U9" s="20">
-        <v>48862</v>
+        <v>40599</v>
       </c>
       <c r="V9" s="20">
-        <v>84112</v>
+        <v>79078</v>
       </c>
       <c r="W9" s="20">
-        <v>129033</v>
+        <v>152346</v>
       </c>
       <c r="X9" s="20">
-        <v>54088</v>
+        <v>69313</v>
       </c>
       <c r="Y9" s="11">
-        <v>65.75</v>
+        <v>54.484999999999999</v>
       </c>
       <c r="Z9" s="11">
-        <v>278.67</v>
+        <v>276.93</v>
       </c>
       <c r="AA9" s="11">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="AB9" s="11">
-        <v>305601</v>
+        <v>318157</v>
       </c>
       <c r="AC9" s="11">
-        <v>405099</v>
+        <v>421743</v>
       </c>
       <c r="AD9" s="11">
         <v>60000</v>
       </c>
       <c r="AE9" s="11">
-        <v>732</v>
+        <v>700.5</v>
       </c>
       <c r="AF9" s="11">
-        <v>652</v>
+        <v>711.5</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" s="10">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="B10" s="11">
-        <v>1.520661</v>
+        <v>2.3409749999999998</v>
       </c>
       <c r="C10" s="11">
-        <v>76542.059815000001</v>
+        <v>67723.616076999999</v>
       </c>
       <c r="D10" s="11">
-        <v>1.3006169999999999</v>
+        <v>1.1937040000000001</v>
       </c>
       <c r="E10" s="11">
-        <v>18161.02189</v>
+        <v>17758.554323</v>
       </c>
       <c r="F10" s="11">
-        <v>9.6300000000000008</v>
+        <v>6.77</v>
       </c>
       <c r="G10" s="11">
-        <v>63.9</v>
+        <v>64.599999999999994</v>
       </c>
       <c r="H10" s="11">
-        <v>13.968859999999999</v>
+        <v>13.388056000000001</v>
       </c>
       <c r="I10" s="11">
-        <v>304.29779300000001</v>
+        <v>269.66826800000001</v>
       </c>
       <c r="J10" s="11">
-        <v>160.55000000000001</v>
+        <v>136.6</v>
       </c>
       <c r="K10" s="11">
-        <v>10.903962</v>
+        <v>11.627488</v>
       </c>
       <c r="L10" s="11">
-        <v>14.352134</v>
+        <v>14.138857</v>
       </c>
       <c r="M10" s="11">
-        <v>44298</v>
+        <v>44449</v>
       </c>
       <c r="N10" s="11">
-        <v>114972</v>
+        <v>125650</v>
       </c>
       <c r="O10" s="11">
-        <v>198846</v>
+        <v>235897</v>
       </c>
       <c r="P10" s="11">
-        <v>88247</v>
+        <v>55807</v>
       </c>
       <c r="Q10" s="20">
-        <v>3585</v>
+        <v>5766</v>
       </c>
       <c r="R10" s="20">
-        <v>35860</v>
+        <v>40857</v>
       </c>
       <c r="S10" s="20">
-        <v>46382</v>
+        <v>57709</v>
       </c>
       <c r="T10" s="20">
-        <v>18934</v>
+        <v>6147</v>
       </c>
       <c r="U10" s="20">
-        <v>40599</v>
+        <v>38632</v>
       </c>
       <c r="V10" s="20">
-        <v>79078</v>
+        <v>84754</v>
       </c>
       <c r="W10" s="20">
-        <v>152346</v>
+        <v>178026</v>
       </c>
       <c r="X10" s="20">
-        <v>69313</v>
+        <v>49659</v>
       </c>
       <c r="Y10" s="11">
-        <v>54.484999999999999</v>
+        <v>43.22</v>
       </c>
       <c r="Z10" s="11">
-        <v>276.93</v>
+        <v>281.19</v>
       </c>
       <c r="AA10" s="11">
-        <v>663</v>
+        <v>736</v>
       </c>
       <c r="AB10" s="11">
-        <v>318157</v>
+        <v>322500</v>
       </c>
       <c r="AC10" s="11">
-        <v>421743</v>
+        <v>427500</v>
       </c>
       <c r="AD10" s="11">
         <v>60000</v>
       </c>
       <c r="AE10" s="11">
-        <v>700.5</v>
+        <v>670</v>
       </c>
       <c r="AF10" s="11">
-        <v>711.5</v>
+        <v>771</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A11" s="10">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="B11" s="11">
-        <v>2.3409749999999998</v>
+        <v>1.541088</v>
       </c>
       <c r="C11" s="11">
-        <v>67723.616076999999</v>
+        <v>65772.980909000005</v>
       </c>
       <c r="D11" s="11">
-        <v>1.1937040000000001</v>
+        <v>0.88603100000000001</v>
       </c>
       <c r="E11" s="11">
-        <v>17758.554323</v>
+        <v>13316.573168999999</v>
       </c>
       <c r="F11" s="11">
-        <v>6.77</v>
+        <v>8.16</v>
       </c>
       <c r="G11" s="11">
-        <v>64.599999999999994</v>
+        <v>64.900000000000006</v>
       </c>
       <c r="H11" s="11">
-        <v>13.388056000000001</v>
+        <v>13.233667000000001</v>
       </c>
       <c r="I11" s="11">
-        <v>269.66826800000001</v>
+        <v>237.379514</v>
       </c>
       <c r="J11" s="11">
-        <v>136.6</v>
+        <v>119.65</v>
       </c>
       <c r="K11" s="11">
-        <v>11.627488</v>
+        <v>12.022000999999999</v>
       </c>
       <c r="L11" s="11">
-        <v>14.138857</v>
+        <v>13.832416</v>
       </c>
       <c r="M11" s="11">
-        <v>44449</v>
+        <v>46650</v>
       </c>
       <c r="N11" s="11">
-        <v>125650</v>
+        <v>111615</v>
       </c>
       <c r="O11" s="11">
-        <v>235897</v>
+        <v>211057</v>
       </c>
       <c r="P11" s="11">
-        <v>55807</v>
+        <v>55699</v>
       </c>
       <c r="Q11" s="20">
-        <v>5766</v>
+        <v>6789</v>
       </c>
       <c r="R11" s="20">
-        <v>40857</v>
+        <v>32187</v>
       </c>
       <c r="S11" s="20">
-        <v>57709</v>
+        <v>56152</v>
       </c>
       <c r="T11" s="20">
-        <v>6147</v>
+        <v>7149</v>
       </c>
       <c r="U11" s="20">
-        <v>38632</v>
+        <v>39736</v>
       </c>
       <c r="V11" s="20">
-        <v>84754</v>
+        <v>79375</v>
       </c>
       <c r="W11" s="20">
-        <v>178026</v>
+        <v>154742</v>
       </c>
       <c r="X11" s="20">
-        <v>49659</v>
+        <v>48549</v>
       </c>
       <c r="Y11" s="11">
-        <v>43.22</v>
+        <v>71.16</v>
       </c>
       <c r="Z11" s="11">
-        <v>281.19</v>
+        <v>282.93</v>
       </c>
       <c r="AA11" s="11">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="AB11" s="11">
-        <v>322500</v>
+        <v>290809</v>
       </c>
       <c r="AC11" s="11">
-        <v>427500</v>
+        <v>385491</v>
       </c>
       <c r="AD11" s="11">
         <v>60000</v>
       </c>
       <c r="AE11" s="11">
-        <v>670</v>
+        <v>694</v>
       </c>
       <c r="AF11" s="11">
-        <v>771</v>
+        <v>704</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A12" s="10">
-        <v>1999</v>
+        <v>2000</v>
       </c>
       <c r="B12" s="11">
-        <v>1.541088</v>
+        <v>2.0877159999999999</v>
       </c>
       <c r="C12" s="11">
-        <v>65772.980909000005</v>
+        <v>62526.498316999998</v>
       </c>
       <c r="D12" s="11">
-        <v>0.88603100000000001</v>
+        <v>0.94496599999999997</v>
       </c>
       <c r="E12" s="11">
-        <v>13316.573168999999</v>
+        <v>12846.517406000001</v>
       </c>
       <c r="F12" s="11">
-        <v>8.16</v>
+        <v>7.41</v>
       </c>
       <c r="G12" s="11">
-        <v>64.900000000000006</v>
+        <v>65.5</v>
       </c>
       <c r="H12" s="11">
-        <v>13.233667000000001</v>
+        <v>15.456422</v>
       </c>
       <c r="I12" s="11">
-        <v>237.379514</v>
+        <v>222.358576</v>
       </c>
       <c r="J12" s="11">
-        <v>119.65</v>
+        <v>142.69999999999999</v>
       </c>
       <c r="K12" s="11">
-        <v>12.022000999999999</v>
+        <v>12.343161</v>
       </c>
       <c r="L12" s="11">
-        <v>13.832416</v>
+        <v>13.897411</v>
       </c>
       <c r="M12" s="11">
-        <v>46650</v>
+        <v>38261</v>
       </c>
       <c r="N12" s="11">
-        <v>111615</v>
+        <v>96047</v>
       </c>
       <c r="O12" s="11">
-        <v>211057</v>
+        <v>238098</v>
       </c>
       <c r="P12" s="11">
-        <v>55699</v>
+        <v>54166</v>
       </c>
       <c r="Q12" s="20">
-        <v>6789</v>
+        <v>4995</v>
       </c>
       <c r="R12" s="20">
-        <v>32187</v>
+        <v>22433</v>
       </c>
       <c r="S12" s="20">
-        <v>56152</v>
+        <v>59059</v>
       </c>
       <c r="T12" s="20">
-        <v>7149</v>
+        <v>9716</v>
       </c>
       <c r="U12" s="20">
-        <v>39736</v>
+        <v>33195</v>
       </c>
       <c r="V12" s="20">
-        <v>79375</v>
+        <v>73589</v>
       </c>
       <c r="W12" s="20">
-        <v>154742</v>
+        <v>178837</v>
       </c>
       <c r="X12" s="20">
-        <v>48549</v>
+        <v>44449</v>
       </c>
       <c r="Y12" s="11">
-        <v>71.16</v>
+        <v>65.349999999999994</v>
       </c>
       <c r="Z12" s="11">
-        <v>282.93</v>
+        <v>284.83999999999997</v>
       </c>
       <c r="AA12" s="11">
-        <v>734</v>
+        <v>889</v>
       </c>
       <c r="AB12" s="11">
-        <v>290809</v>
+        <v>297732</v>
       </c>
       <c r="AC12" s="11">
-        <v>385491</v>
+        <v>394668</v>
       </c>
       <c r="AD12" s="11">
         <v>60000</v>
       </c>
       <c r="AE12" s="11">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="AF12" s="11">
-        <v>704</v>
+        <v>759</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A13" s="10">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="B13" s="11">
-        <v>2.0877159999999999</v>
+        <v>1.0578719999999999</v>
       </c>
       <c r="C13" s="11">
-        <v>62526.498316999998</v>
+        <v>34617.503272000002</v>
       </c>
       <c r="D13" s="11">
-        <v>0.94496599999999997</v>
+        <v>0.56989699999999999</v>
       </c>
       <c r="E13" s="11">
-        <v>12846.517406000001</v>
+        <v>7553.7379190000001</v>
       </c>
       <c r="F13" s="11">
-        <v>7.41</v>
+        <v>4.29</v>
       </c>
       <c r="G13" s="11">
-        <v>65.5</v>
+        <v>65</v>
       </c>
       <c r="H13" s="11">
-        <v>15.456422</v>
+        <v>13.018592999999999</v>
       </c>
       <c r="I13" s="11">
-        <v>222.358576</v>
+        <v>214.22200000000001</v>
       </c>
       <c r="J13" s="11">
-        <v>142.69999999999999</v>
+        <v>165.35</v>
       </c>
       <c r="K13" s="11">
-        <v>12.343161</v>
+        <v>12.270602999999999</v>
       </c>
       <c r="L13" s="11">
-        <v>13.897411</v>
+        <v>13.90582</v>
       </c>
       <c r="M13" s="11">
-        <v>38261</v>
+        <v>34475</v>
       </c>
       <c r="N13" s="11">
-        <v>96047</v>
+        <v>99924</v>
       </c>
       <c r="O13" s="11">
-        <v>238098</v>
+        <v>246513</v>
       </c>
       <c r="P13" s="11">
-        <v>54166</v>
+        <v>83805</v>
       </c>
       <c r="Q13" s="20">
-        <v>4995</v>
+        <v>2777</v>
       </c>
       <c r="R13" s="20">
-        <v>22433</v>
+        <v>23231</v>
       </c>
       <c r="S13" s="20">
-        <v>59059</v>
+        <v>64883</v>
       </c>
       <c r="T13" s="20">
-        <v>9716</v>
+        <v>21061</v>
       </c>
       <c r="U13" s="20">
-        <v>33195</v>
+        <v>31588</v>
       </c>
       <c r="V13" s="20">
-        <v>73589</v>
+        <v>76640</v>
       </c>
       <c r="W13" s="20">
-        <v>178837</v>
+        <v>181446</v>
       </c>
       <c r="X13" s="20">
-        <v>44449</v>
+        <v>62739</v>
       </c>
       <c r="Y13" s="11">
-        <v>65.349999999999994</v>
+        <v>58.24</v>
       </c>
       <c r="Z13" s="11">
-        <v>284.83999999999997</v>
+        <v>286.76</v>
       </c>
       <c r="AA13" s="11">
-        <v>889</v>
+        <v>895.5</v>
       </c>
       <c r="AB13" s="11">
-        <v>297732</v>
+        <v>313040</v>
       </c>
       <c r="AC13" s="11">
-        <v>394668</v>
+        <v>414960</v>
       </c>
       <c r="AD13" s="11">
         <v>60000</v>
       </c>
       <c r="AE13" s="11">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="AF13" s="11">
-        <v>759</v>
+        <v>666</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="B14" s="11">
-        <v>1.0578719999999999</v>
+        <v>1.6741680000000001</v>
       </c>
       <c r="C14" s="11">
-        <v>34617.503272000002</v>
+        <v>49141.771323000001</v>
       </c>
       <c r="D14" s="11">
-        <v>0.56989699999999999</v>
+        <v>0.80114600000000002</v>
       </c>
       <c r="E14" s="11">
-        <v>7553.7379190000001</v>
+        <v>9126.0629069999995</v>
       </c>
       <c r="F14" s="11">
-        <v>4.29</v>
+        <v>6.89</v>
       </c>
       <c r="G14" s="11">
-        <v>65</v>
+        <v>65.3</v>
       </c>
       <c r="H14" s="11">
-        <v>13.018592999999999</v>
+        <v>12.096083999999999</v>
       </c>
       <c r="I14" s="11">
-        <v>214.22200000000001</v>
+        <v>207.625711</v>
       </c>
       <c r="J14" s="11">
-        <v>165.35</v>
+        <v>131.05000000000001</v>
       </c>
       <c r="K14" s="11">
-        <v>12.270602999999999</v>
+        <v>12.464226</v>
       </c>
       <c r="L14" s="11">
-        <v>13.90582</v>
+        <v>13.742813999999999</v>
       </c>
       <c r="M14" s="11">
-        <v>34475</v>
+        <v>59041</v>
       </c>
       <c r="N14" s="11">
-        <v>99924</v>
+        <v>107285</v>
       </c>
       <c r="O14" s="11">
-        <v>246513</v>
+        <v>259254</v>
       </c>
       <c r="P14" s="11">
-        <v>83805</v>
+        <v>36359</v>
       </c>
       <c r="Q14" s="20">
-        <v>2777</v>
+        <v>8610</v>
       </c>
       <c r="R14" s="20">
-        <v>23231</v>
+        <v>22827</v>
       </c>
       <c r="S14" s="20">
-        <v>64883</v>
+        <v>68313</v>
       </c>
       <c r="T14" s="20">
-        <v>21061</v>
+        <v>6418</v>
       </c>
       <c r="U14" s="20">
-        <v>31588</v>
+        <v>50378</v>
       </c>
       <c r="V14" s="20">
-        <v>76640</v>
+        <v>84383</v>
       </c>
       <c r="W14" s="20">
-        <v>181446</v>
+        <v>190868</v>
       </c>
       <c r="X14" s="20">
-        <v>62739</v>
+        <v>29935</v>
       </c>
       <c r="Y14" s="11">
-        <v>58.24</v>
+        <v>55.03</v>
       </c>
       <c r="Z14" s="11">
-        <v>286.76</v>
+        <v>286.39</v>
       </c>
       <c r="AA14" s="11">
-        <v>895.5</v>
+        <v>948.6</v>
       </c>
       <c r="AB14" s="11">
-        <v>313040</v>
+        <v>319232</v>
       </c>
       <c r="AC14" s="11">
-        <v>414960</v>
+        <v>423168</v>
       </c>
       <c r="AD14" s="11">
         <v>60000</v>
       </c>
       <c r="AE14" s="11">
-        <v>698</v>
+        <v>660</v>
       </c>
       <c r="AF14" s="11">
-        <v>666</v>
+        <v>568</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="B15" s="11">
-        <v>1.6741680000000001</v>
+        <v>1.6867179999999999</v>
       </c>
       <c r="C15" s="11">
-        <v>49141.771323000001</v>
+        <v>59774.328823999997</v>
       </c>
       <c r="D15" s="11">
-        <v>0.80114600000000002</v>
+        <v>1.0799110000000001</v>
       </c>
       <c r="E15" s="11">
-        <v>9126.0629069999995</v>
+        <v>14649.845083</v>
       </c>
       <c r="F15" s="11">
-        <v>6.89</v>
+        <v>4.21</v>
       </c>
       <c r="G15" s="11">
-        <v>65.3</v>
+        <v>66</v>
       </c>
       <c r="H15" s="11">
-        <v>12.096083999999999</v>
+        <v>11.827598</v>
       </c>
       <c r="I15" s="11">
-        <v>207.625711</v>
+        <v>203.330082</v>
       </c>
       <c r="J15" s="11">
-        <v>131.05000000000001</v>
+        <v>179.55</v>
       </c>
       <c r="K15" s="11">
-        <v>12.464226</v>
+        <v>12.890366999999999</v>
       </c>
       <c r="L15" s="11">
-        <v>13.742813999999999</v>
+        <v>13.612512000000001</v>
       </c>
       <c r="M15" s="11">
-        <v>59041</v>
+        <v>50147</v>
       </c>
       <c r="N15" s="11">
-        <v>107285</v>
+        <v>94176</v>
       </c>
       <c r="O15" s="11">
-        <v>259254</v>
+        <v>271690</v>
       </c>
       <c r="P15" s="11">
-        <v>36359</v>
+        <v>51159</v>
       </c>
       <c r="Q15" s="20">
-        <v>8610</v>
+        <v>5768</v>
       </c>
       <c r="R15" s="20">
-        <v>22827</v>
+        <v>21363</v>
       </c>
       <c r="S15" s="20">
-        <v>68313</v>
+        <v>72330</v>
       </c>
       <c r="T15" s="20">
-        <v>6418</v>
+        <v>12654</v>
       </c>
       <c r="U15" s="20">
-        <v>50378</v>
+        <v>44338</v>
       </c>
       <c r="V15" s="20">
-        <v>84383</v>
+        <v>72778</v>
       </c>
       <c r="W15" s="20">
-        <v>190868</v>
+        <v>199232</v>
       </c>
       <c r="X15" s="20">
-        <v>29935</v>
+        <v>38482</v>
       </c>
       <c r="Y15" s="11">
-        <v>55.03</v>
+        <v>61.83</v>
       </c>
       <c r="Z15" s="11">
-        <v>286.39</v>
+        <v>287.92</v>
       </c>
       <c r="AA15" s="11">
-        <v>948.6</v>
+        <v>1001.7</v>
       </c>
       <c r="AB15" s="11">
-        <v>319232</v>
+        <v>135751</v>
       </c>
       <c r="AC15" s="11">
-        <v>423168</v>
+        <v>170000</v>
       </c>
       <c r="AD15" s="11">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="AE15" s="11">
-        <v>660</v>
+        <v>1305</v>
       </c>
       <c r="AF15" s="11">
-        <v>568</v>
+        <v>881</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="B16" s="11">
-        <v>1.6867179999999999</v>
+        <v>2.9381520000000001</v>
       </c>
       <c r="C16" s="11">
-        <v>59774.328823999997</v>
+        <v>85911.146984999999</v>
       </c>
       <c r="D16" s="11">
-        <v>1.0799110000000001</v>
+        <v>0.746224</v>
       </c>
       <c r="E16" s="11">
-        <v>14649.845083</v>
+        <v>10891.443332999999</v>
       </c>
       <c r="F16" s="11">
-        <v>4.21</v>
+        <v>12.09</v>
       </c>
       <c r="G16" s="11">
-        <v>66</v>
+        <v>64.099999999999994</v>
       </c>
       <c r="H16" s="11">
-        <v>11.827598</v>
+        <v>12.036407000000001</v>
       </c>
       <c r="I16" s="11">
-        <v>203.330082</v>
+        <v>204.94497699999999</v>
       </c>
       <c r="J16" s="11">
-        <v>179.55</v>
+        <v>200.2</v>
       </c>
       <c r="K16" s="11">
-        <v>12.890366999999999</v>
+        <v>12.904496999999999</v>
       </c>
       <c r="L16" s="11">
-        <v>13.612512000000001</v>
+        <v>13.476324</v>
       </c>
       <c r="M16" s="11">
-        <v>50147</v>
+        <v>43355</v>
       </c>
       <c r="N16" s="11">
-        <v>94176</v>
+        <v>99758</v>
       </c>
       <c r="O16" s="11">
-        <v>271690</v>
+        <v>223648</v>
       </c>
       <c r="P16" s="11">
-        <v>51159</v>
+        <v>30480</v>
       </c>
       <c r="Q16" s="20">
-        <v>5768</v>
+        <v>4258</v>
       </c>
       <c r="R16" s="20">
-        <v>21363</v>
+        <v>18706</v>
       </c>
       <c r="S16" s="20">
-        <v>72330</v>
+        <v>63318</v>
       </c>
       <c r="T16" s="20">
-        <v>12654</v>
+        <v>4934</v>
       </c>
       <c r="U16" s="20">
-        <v>44338</v>
+        <v>39074</v>
       </c>
       <c r="V16" s="20">
-        <v>72778</v>
+        <v>80969</v>
       </c>
       <c r="W16" s="20">
-        <v>199232</v>
+        <v>160282</v>
       </c>
       <c r="X16" s="20">
-        <v>38482</v>
+        <v>25542</v>
       </c>
       <c r="Y16" s="11">
-        <v>61.83</v>
+        <v>64.02</v>
       </c>
       <c r="Z16" s="11">
-        <v>287.92</v>
+        <v>287.69</v>
       </c>
       <c r="AA16" s="11">
-        <v>1001.7</v>
+        <v>1054.8</v>
       </c>
       <c r="AB16" s="11">
-        <v>135751</v>
+        <v>146415</v>
       </c>
       <c r="AC16" s="11">
-        <v>170000</v>
+        <v>173085</v>
       </c>
       <c r="AD16" s="11">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="AE16" s="11">
-        <v>1305</v>
+        <v>1550</v>
       </c>
       <c r="AF16" s="11">
-        <v>881</v>
+        <v>953</v>
       </c>
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A17" s="10">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="B17" s="11">
-        <v>2.9381520000000001</v>
+        <v>2.3412679999999999</v>
       </c>
       <c r="C17" s="11">
-        <v>85911.146984999999</v>
+        <v>75117.357071000006</v>
       </c>
       <c r="D17" s="11">
-        <v>0.746224</v>
+        <v>0.80249000000000004</v>
       </c>
       <c r="E17" s="11">
-        <v>10891.443332999999</v>
+        <v>9376.1489309999997</v>
       </c>
       <c r="F17" s="11">
-        <v>12.09</v>
+        <v>12.87</v>
       </c>
       <c r="G17" s="11">
-        <v>64.099999999999994</v>
+        <v>65.7</v>
       </c>
       <c r="H17" s="11">
-        <v>12.036407000000001</v>
+        <v>12.077712</v>
       </c>
       <c r="I17" s="11">
-        <v>204.94497699999999</v>
+        <v>190.20649399999999</v>
       </c>
       <c r="J17" s="11">
-        <v>200.2</v>
+        <v>229.4</v>
       </c>
       <c r="K17" s="11">
-        <v>12.904496999999999</v>
+        <v>12.642844999999999</v>
       </c>
       <c r="L17" s="11">
-        <v>13.476324</v>
+        <v>13.40612</v>
       </c>
       <c r="M17" s="11">
-        <v>43355</v>
+        <v>74245</v>
       </c>
       <c r="N17" s="11">
-        <v>99758</v>
+        <v>98930</v>
       </c>
       <c r="O17" s="11">
-        <v>223648</v>
+        <v>249797</v>
       </c>
       <c r="P17" s="11">
-        <v>30480</v>
+        <v>40351</v>
       </c>
       <c r="Q17" s="20">
-        <v>4258</v>
+        <v>12302</v>
       </c>
       <c r="R17" s="20">
-        <v>18706</v>
+        <v>20713</v>
       </c>
       <c r="S17" s="20">
-        <v>63318</v>
+        <v>70953</v>
       </c>
       <c r="T17" s="20">
-        <v>4934</v>
+        <v>10329</v>
       </c>
       <c r="U17" s="20">
-        <v>39074</v>
+        <v>61812</v>
       </c>
       <c r="V17" s="20">
-        <v>80969</v>
+        <v>78148</v>
       </c>
       <c r="W17" s="20">
-        <v>160282</v>
+        <v>178771</v>
       </c>
       <c r="X17" s="20">
-        <v>25542</v>
+        <v>30015</v>
       </c>
       <c r="Y17" s="11">
-        <v>64.02</v>
+        <v>49.78</v>
       </c>
       <c r="Z17" s="11">
-        <v>287.69</v>
+        <v>289.54000000000002</v>
       </c>
       <c r="AA17" s="11">
-        <v>1054.8</v>
+        <v>1107.9000000000001</v>
       </c>
       <c r="AB17" s="11">
-        <v>146415</v>
+        <v>247610</v>
       </c>
       <c r="AC17" s="11">
-        <v>173085</v>
+        <v>356690</v>
       </c>
       <c r="AD17" s="11">
-        <v>60000</v>
+        <v>58600</v>
       </c>
       <c r="AE17" s="11">
-        <v>1550</v>
+        <v>780</v>
       </c>
       <c r="AF17" s="11">
-        <v>953</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A18" s="10">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="B18" s="11">
-        <v>2.3412679999999999</v>
+        <v>2.440067</v>
       </c>
       <c r="C18" s="11">
-        <v>75117.357071000006</v>
+        <v>71961.043132999999</v>
       </c>
       <c r="D18" s="11">
-        <v>0.80249000000000004</v>
+        <v>0.757046</v>
       </c>
       <c r="E18" s="11">
-        <v>9376.1489309999997</v>
+        <v>9957.9837509999998</v>
       </c>
       <c r="F18" s="11">
-        <v>12.87</v>
+        <v>17.510000000000002</v>
       </c>
       <c r="G18" s="11">
-        <v>65.7</v>
+        <v>65.900000000000006</v>
       </c>
       <c r="H18" s="11">
-        <v>12.077712</v>
+        <v>13.811404</v>
       </c>
       <c r="I18" s="11">
-        <v>190.20649399999999</v>
+        <v>190.17796799999999</v>
       </c>
       <c r="J18" s="11">
-        <v>229.4</v>
+        <v>237.85</v>
       </c>
       <c r="K18" s="11">
-        <v>12.642844999999999</v>
+        <v>12.779068000000001</v>
       </c>
       <c r="L18" s="11">
-        <v>13.40612</v>
+        <v>13.453433</v>
       </c>
       <c r="M18" s="11">
-        <v>74245</v>
+        <v>47671</v>
       </c>
       <c r="N18" s="11">
-        <v>98930</v>
+        <v>85294</v>
       </c>
       <c r="O18" s="11">
-        <v>249797</v>
+        <v>260220</v>
       </c>
       <c r="P18" s="11">
-        <v>40351</v>
+        <v>38812</v>
       </c>
       <c r="Q18" s="20">
-        <v>12302</v>
+        <v>5093</v>
       </c>
       <c r="R18" s="20">
-        <v>20713</v>
+        <v>17478</v>
       </c>
       <c r="S18" s="20">
-        <v>70953</v>
+        <v>69508</v>
       </c>
       <c r="T18" s="20">
-        <v>10329</v>
+        <v>3658</v>
       </c>
       <c r="U18" s="20">
-        <v>61812</v>
+        <v>42562</v>
       </c>
       <c r="V18" s="20">
-        <v>78148</v>
+        <v>67756</v>
       </c>
       <c r="W18" s="20">
-        <v>178771</v>
+        <v>190650</v>
       </c>
       <c r="X18" s="20">
-        <v>30015</v>
+        <v>35150</v>
       </c>
       <c r="Y18" s="11">
-        <v>49.78</v>
+        <v>64.63</v>
       </c>
       <c r="Z18" s="11">
-        <v>289.54000000000002</v>
+        <v>289.89999999999998</v>
       </c>
       <c r="AA18" s="11">
-        <v>1107.9000000000001</v>
+        <v>1161</v>
       </c>
       <c r="AB18" s="11">
-        <v>247610</v>
+        <v>154746</v>
       </c>
       <c r="AC18" s="11">
-        <v>356690</v>
+        <v>210139</v>
       </c>
       <c r="AD18" s="11">
-        <v>58600</v>
+        <v>28532</v>
       </c>
       <c r="AE18" s="11">
-        <v>780</v>
+        <v>731.5</v>
       </c>
       <c r="AF18" s="11">
-        <v>1250</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="B19" s="11">
-        <v>2.440067</v>
+        <v>1.7032989999999999</v>
       </c>
       <c r="C19" s="11">
-        <v>71961.043132999999</v>
+        <v>60482.175635</v>
       </c>
       <c r="D19" s="11">
-        <v>0.757046</v>
+        <v>0.93225199999999997</v>
       </c>
       <c r="E19" s="11">
-        <v>9957.9837509999998</v>
+        <v>11118.45455</v>
       </c>
       <c r="F19" s="11">
-        <v>17.510000000000002</v>
+        <v>10.119999999999999</v>
       </c>
       <c r="G19" s="11">
-        <v>65.900000000000006</v>
+        <v>65.3</v>
       </c>
       <c r="H19" s="11">
-        <v>13.811404</v>
+        <v>11.406019000000001</v>
       </c>
       <c r="I19" s="11">
-        <v>190.17796799999999</v>
+        <v>187.17006000000001</v>
       </c>
       <c r="J19" s="11">
-        <v>237.85</v>
+        <v>281.95</v>
       </c>
       <c r="K19" s="11">
-        <v>12.779068000000001</v>
+        <v>12.744325999999999</v>
       </c>
       <c r="L19" s="11">
-        <v>13.453433</v>
+        <v>13.444872</v>
       </c>
       <c r="M19" s="11">
-        <v>47671</v>
+        <v>63678</v>
       </c>
       <c r="N19" s="11">
-        <v>85294</v>
+        <v>87179</v>
       </c>
       <c r="O19" s="11">
-        <v>260220</v>
+        <v>304871</v>
       </c>
       <c r="P19" s="11">
-        <v>38812</v>
+        <v>52643</v>
       </c>
       <c r="Q19" s="20">
-        <v>5093</v>
+        <v>10228</v>
       </c>
       <c r="R19" s="20">
-        <v>17478</v>
+        <v>22307</v>
       </c>
       <c r="S19" s="20">
-        <v>69508</v>
+        <v>77649</v>
       </c>
       <c r="T19" s="20">
-        <v>3658</v>
+        <v>7504</v>
       </c>
       <c r="U19" s="20">
-        <v>42562</v>
+        <v>53339</v>
       </c>
       <c r="V19" s="20">
-        <v>67756</v>
+        <v>64816</v>
       </c>
       <c r="W19" s="20">
-        <v>190650</v>
+        <v>227065</v>
       </c>
       <c r="X19" s="20">
-        <v>35150</v>
+        <v>45134</v>
       </c>
       <c r="Y19" s="11">
-        <v>64.63</v>
+        <v>62.58</v>
       </c>
       <c r="Z19" s="11">
-        <v>289.89999999999998</v>
+        <v>287.98</v>
       </c>
       <c r="AA19" s="11">
-        <v>1161</v>
+        <v>1214.0999999999999</v>
       </c>
       <c r="AB19" s="11">
-        <v>154746</v>
+        <v>278251</v>
       </c>
       <c r="AC19" s="11">
-        <v>210139</v>
+        <v>302664</v>
       </c>
       <c r="AD19" s="11">
-        <v>28532</v>
+        <v>51245</v>
       </c>
       <c r="AE19" s="11">
-        <v>731.5</v>
+        <v>750</v>
       </c>
       <c r="AF19" s="11">
-        <v>1060</v>
+        <v>786</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A20" s="10">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="B20" s="11">
-        <v>1.7032989999999999</v>
+        <v>1.962515</v>
       </c>
       <c r="C20" s="11">
-        <v>60482.175635</v>
+        <v>75502.947528999997</v>
       </c>
       <c r="D20" s="11">
-        <v>0.93225199999999997</v>
+        <v>0.71910099999999999</v>
       </c>
       <c r="E20" s="11">
-        <v>11118.45455</v>
+        <v>10084.609780000001</v>
       </c>
       <c r="F20" s="11">
-        <v>10.119999999999999</v>
+        <v>9.86</v>
       </c>
       <c r="G20" s="11">
-        <v>65.3</v>
+        <v>65</v>
       </c>
       <c r="H20" s="11">
-        <v>11.406019000000001</v>
+        <v>12.741701000000001</v>
       </c>
       <c r="I20" s="11">
-        <v>187.17006000000001</v>
+        <v>188.15249900000001</v>
       </c>
       <c r="J20" s="11">
-        <v>281.95</v>
+        <v>424.5</v>
       </c>
       <c r="K20" s="11">
-        <v>12.744325999999999</v>
+        <v>12.624536000000001</v>
       </c>
       <c r="L20" s="11">
-        <v>13.444872</v>
+        <v>13.29965</v>
       </c>
       <c r="M20" s="11">
-        <v>63678</v>
+        <v>68064</v>
       </c>
       <c r="N20" s="11">
-        <v>87179</v>
+        <v>72241</v>
       </c>
       <c r="O20" s="11">
-        <v>304871</v>
+        <v>289100</v>
       </c>
       <c r="P20" s="11">
-        <v>52643</v>
+        <v>63160</v>
       </c>
       <c r="Q20" s="20">
-        <v>10228</v>
+        <v>12390</v>
       </c>
       <c r="R20" s="20">
-        <v>22307</v>
+        <v>24086</v>
       </c>
       <c r="S20" s="20">
-        <v>77649</v>
+        <v>79372</v>
       </c>
       <c r="T20" s="20">
-        <v>7504</v>
+        <v>10840</v>
       </c>
       <c r="U20" s="20">
-        <v>53339</v>
+        <v>55666</v>
       </c>
       <c r="V20" s="20">
-        <v>64816</v>
+        <v>47914</v>
       </c>
       <c r="W20" s="20">
-        <v>227065</v>
+        <v>209650</v>
       </c>
       <c r="X20" s="20">
-        <v>45134</v>
+        <v>52311</v>
       </c>
       <c r="Y20" s="11">
-        <v>62.58</v>
+        <v>66.95</v>
       </c>
       <c r="Z20" s="11">
-        <v>287.98</v>
+        <v>288.52</v>
       </c>
       <c r="AA20" s="11">
-        <v>1214.0999999999999</v>
+        <v>1267.2</v>
       </c>
       <c r="AB20" s="11">
-        <v>278251</v>
+        <v>279173</v>
       </c>
       <c r="AC20" s="11">
-        <v>302664</v>
+        <v>329294</v>
       </c>
       <c r="AD20" s="11">
-        <v>51245</v>
+        <v>56048</v>
       </c>
       <c r="AE20" s="11">
-        <v>750</v>
+        <v>672</v>
       </c>
       <c r="AF20" s="11">
-        <v>786</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A21" s="10">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="B21" s="11">
-        <v>1.962515</v>
+        <v>2.1018919999999999</v>
       </c>
       <c r="C21" s="11">
-        <v>75502.947528999997</v>
+        <v>65980.949995000003</v>
       </c>
       <c r="D21" s="11">
-        <v>0.71910099999999999</v>
+        <v>0.95246600000000003</v>
       </c>
       <c r="E21" s="11">
-        <v>10084.609780000001</v>
+        <v>12954.526943999999</v>
       </c>
       <c r="F21" s="11">
-        <v>9.86</v>
+        <v>8.68</v>
       </c>
       <c r="G21" s="11">
-        <v>65</v>
+        <v>66.400000000000006</v>
       </c>
       <c r="H21" s="11">
-        <v>12.741701000000001</v>
+        <v>12.493766000000001</v>
       </c>
       <c r="I21" s="11">
-        <v>188.15249900000001</v>
+        <v>205.58075099999999</v>
       </c>
       <c r="J21" s="11">
-        <v>424.5</v>
+        <v>257.39999999999998</v>
       </c>
       <c r="K21" s="11">
-        <v>12.624536000000001</v>
+        <v>13.963621</v>
       </c>
       <c r="L21" s="11">
-        <v>13.29965</v>
+        <v>13.161011</v>
       </c>
       <c r="M21" s="11">
-        <v>68064</v>
+        <v>59583</v>
       </c>
       <c r="N21" s="11">
-        <v>72241</v>
+        <v>52225</v>
       </c>
       <c r="O21" s="11">
-        <v>289100</v>
+        <v>281741</v>
       </c>
       <c r="P21" s="11">
-        <v>63160</v>
+        <v>91721</v>
       </c>
       <c r="Q21" s="20">
-        <v>12390</v>
+        <v>5263</v>
       </c>
       <c r="R21" s="20">
-        <v>24086</v>
+        <v>8002</v>
       </c>
       <c r="S21" s="20">
-        <v>79372</v>
+        <v>78843</v>
       </c>
       <c r="T21" s="20">
-        <v>10840</v>
+        <v>25761</v>
       </c>
       <c r="U21" s="20">
-        <v>55666</v>
+        <v>54320</v>
       </c>
       <c r="V21" s="20">
-        <v>47914</v>
+        <v>44219</v>
       </c>
       <c r="W21" s="20">
-        <v>209650</v>
+        <v>202847</v>
       </c>
       <c r="X21" s="20">
-        <v>52311</v>
+        <v>65958</v>
       </c>
       <c r="Y21" s="11">
-        <v>66.95</v>
+        <v>68.44</v>
       </c>
       <c r="Z21" s="11">
-        <v>288.52</v>
+        <v>290.69</v>
       </c>
       <c r="AA21" s="11">
-        <v>1267.2</v>
+        <v>1320.3</v>
       </c>
       <c r="AB21" s="11">
-        <v>279173</v>
+        <v>320116</v>
       </c>
       <c r="AC21" s="11">
-        <v>329294</v>
+        <v>305475</v>
       </c>
       <c r="AD21" s="11">
-        <v>56048</v>
+        <v>58688</v>
       </c>
       <c r="AE21" s="11">
-        <v>672</v>
+        <v>594</v>
       </c>
       <c r="AF21" s="11">
-        <v>1006</v>
+        <v>913</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A22" s="10">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="B22" s="11">
-        <v>2.1018919999999999</v>
+        <v>3.3261180000000001</v>
       </c>
       <c r="C22" s="11">
-        <v>65980.949995000003</v>
+        <v>99468.967994999999</v>
       </c>
       <c r="D22" s="11">
-        <v>0.95246600000000003</v>
+        <v>1.223433</v>
       </c>
       <c r="E22" s="11">
-        <v>12954.526943999999</v>
+        <v>17163.732752</v>
       </c>
       <c r="F22" s="11">
-        <v>8.68</v>
+        <v>6.67</v>
       </c>
       <c r="G22" s="11">
-        <v>66.400000000000006</v>
+        <v>65.900000000000006</v>
       </c>
       <c r="H22" s="11">
-        <v>12.493766000000001</v>
+        <v>9.9783530000000003</v>
       </c>
       <c r="I22" s="11">
-        <v>205.58075099999999</v>
+        <v>189.991829</v>
       </c>
       <c r="J22" s="11">
-        <v>257.39999999999998</v>
+        <v>287.95</v>
       </c>
       <c r="K22" s="11">
-        <v>13.963621</v>
+        <v>13.449085</v>
       </c>
       <c r="L22" s="11">
-        <v>13.161011</v>
+        <v>13.248702</v>
       </c>
       <c r="M22" s="11">
-        <v>59583</v>
+        <v>70923</v>
       </c>
       <c r="N22" s="11">
-        <v>52225</v>
+        <v>108562</v>
       </c>
       <c r="O22" s="11">
-        <v>281741</v>
+        <v>274027</v>
       </c>
       <c r="P22" s="11">
-        <v>91721</v>
+        <v>85807</v>
       </c>
       <c r="Q22" s="20">
-        <v>5263</v>
+        <v>11164</v>
       </c>
       <c r="R22" s="20">
-        <v>8002</v>
+        <v>27858</v>
       </c>
       <c r="S22" s="20">
-        <v>78843</v>
+        <v>80127</v>
       </c>
       <c r="T22" s="20">
-        <v>25761</v>
+        <v>24877</v>
       </c>
       <c r="U22" s="20">
-        <v>54320</v>
+        <v>59759</v>
       </c>
       <c r="V22" s="20">
-        <v>44219</v>
+        <v>80695</v>
       </c>
       <c r="W22" s="20">
-        <v>202847</v>
+        <v>193863</v>
       </c>
       <c r="X22" s="20">
-        <v>65958</v>
+        <v>60927</v>
       </c>
       <c r="Y22" s="11">
-        <v>68.44</v>
+        <v>77.77</v>
       </c>
       <c r="Z22" s="11">
-        <v>290.69</v>
+        <v>291.68</v>
       </c>
       <c r="AA22" s="11">
-        <v>1320.3</v>
+        <v>1373.4</v>
       </c>
       <c r="AB22" s="11">
-        <v>320116</v>
+        <v>304937</v>
       </c>
       <c r="AC22" s="11">
-        <v>305475</v>
+        <v>282082</v>
       </c>
       <c r="AD22" s="11">
-        <v>58688</v>
+        <v>56883</v>
       </c>
       <c r="AE22" s="11">
-        <v>594</v>
+        <v>650</v>
       </c>
       <c r="AF22" s="11">
-        <v>913</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="B23" s="11">
-        <v>3.3261180000000001</v>
+        <v>3.4064709999999998</v>
       </c>
       <c r="C23" s="11">
-        <v>99468.967994999999</v>
+        <v>112556.338865</v>
       </c>
       <c r="D23" s="11">
-        <v>1.223433</v>
+        <v>1.3107200000000001</v>
       </c>
       <c r="E23" s="11">
-        <v>17163.732752</v>
+        <v>16946.990851999999</v>
       </c>
       <c r="F23" s="11">
-        <v>6.67</v>
+        <v>5.27</v>
       </c>
       <c r="G23" s="11">
-        <v>65.900000000000006</v>
+        <v>66.599999999999994</v>
       </c>
       <c r="H23" s="11">
-        <v>9.9783530000000003</v>
+        <v>11.495088000000001</v>
       </c>
       <c r="I23" s="11">
-        <v>189.991829</v>
+        <v>162.32168899999999</v>
       </c>
       <c r="J23" s="11">
-        <v>287.95</v>
+        <v>409.3</v>
       </c>
       <c r="K23" s="11">
-        <v>13.449085</v>
+        <v>13.415609</v>
       </c>
       <c r="L23" s="11">
-        <v>13.248702</v>
+        <v>13.338027</v>
       </c>
       <c r="M23" s="11">
-        <v>70923</v>
+        <v>57678</v>
       </c>
       <c r="N23" s="11">
-        <v>108562</v>
+        <v>103186</v>
       </c>
       <c r="O23" s="11">
-        <v>274027</v>
+        <v>302267</v>
       </c>
       <c r="P23" s="11">
-        <v>85807</v>
+        <v>54374</v>
       </c>
       <c r="Q23" s="20">
-        <v>11164</v>
+        <v>3515</v>
       </c>
       <c r="R23" s="20">
-        <v>27858</v>
+        <v>28107</v>
       </c>
       <c r="S23" s="20">
-        <v>80127</v>
+        <v>84791</v>
       </c>
       <c r="T23" s="20">
-        <v>24877</v>
+        <v>12600</v>
       </c>
       <c r="U23" s="20">
-        <v>59759</v>
+        <v>54157</v>
       </c>
       <c r="V23" s="20">
-        <v>80695</v>
+        <v>75069</v>
       </c>
       <c r="W23" s="20">
-        <v>193863</v>
+        <v>217445</v>
       </c>
       <c r="X23" s="20">
-        <v>60927</v>
+        <v>41771</v>
       </c>
       <c r="Y23" s="11">
-        <v>77.77</v>
+        <v>69.900000000000006</v>
       </c>
       <c r="Z23" s="11">
-        <v>291.68</v>
+        <v>290.77</v>
       </c>
       <c r="AA23" s="11">
-        <v>1373.4</v>
+        <v>1426.5</v>
       </c>
       <c r="AB23" s="11">
-        <v>304937</v>
+        <v>267814</v>
       </c>
       <c r="AC23" s="11">
-        <v>282082</v>
+        <v>77104</v>
       </c>
       <c r="AD23" s="11">
-        <v>56883</v>
+        <v>25649</v>
       </c>
       <c r="AE23" s="11">
-        <v>650</v>
+        <v>1172</v>
       </c>
       <c r="AF23" s="11">
-        <v>1380</v>
+        <v>778.75</v>
       </c>
     </row>
     <row r="24" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A24" s="10">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="B24" s="11">
-        <v>3.4064709999999998</v>
+        <v>2.1562540000000001</v>
       </c>
       <c r="C24" s="11">
-        <v>112556.338865</v>
+        <v>74319.765438999995</v>
       </c>
       <c r="D24" s="11">
-        <v>1.3107200000000001</v>
+        <v>1.0396719999999999</v>
       </c>
       <c r="E24" s="11">
-        <v>16946.990851999999</v>
+        <v>15146.924349000001</v>
       </c>
       <c r="F24" s="11">
-        <v>5.27</v>
+        <v>6.04</v>
       </c>
       <c r="G24" s="11">
-        <v>66.599999999999994</v>
+        <v>67.099999999999994</v>
       </c>
       <c r="H24" s="11">
-        <v>11.495088000000001</v>
+        <v>10.57526</v>
       </c>
       <c r="I24" s="11">
-        <v>162.32168899999999</v>
+        <v>174.76034200000001</v>
       </c>
       <c r="J24" s="11">
-        <v>409.3</v>
+        <v>433.75</v>
       </c>
       <c r="K24" s="11">
-        <v>13.415609</v>
+        <v>13.390751</v>
       </c>
       <c r="L24" s="11">
-        <v>13.338027</v>
+        <v>13.349034</v>
       </c>
       <c r="M24" s="11">
-        <v>57678</v>
+        <v>57595</v>
       </c>
       <c r="N24" s="11">
-        <v>103186</v>
+        <v>82114.5</v>
       </c>
       <c r="O24" s="11">
-        <v>302267</v>
+        <v>299594.5</v>
       </c>
       <c r="P24" s="11">
-        <v>54374</v>
+        <v>51376.5</v>
       </c>
       <c r="Q24" s="20">
-        <v>3515</v>
+        <v>3746.5</v>
       </c>
       <c r="R24" s="20">
-        <v>28107</v>
+        <v>23490.5</v>
       </c>
       <c r="S24" s="20">
-        <v>84791</v>
+        <v>75587</v>
       </c>
       <c r="T24" s="20">
-        <v>12600</v>
+        <v>12867.5</v>
       </c>
       <c r="U24" s="20">
-        <v>54157</v>
+        <v>53843.5</v>
       </c>
       <c r="V24" s="20">
-        <v>75069</v>
+        <v>58619.5</v>
       </c>
       <c r="W24" s="20">
-        <v>217445</v>
+        <v>223968.5</v>
       </c>
       <c r="X24" s="20">
-        <v>41771</v>
+        <v>38508</v>
       </c>
       <c r="Y24" s="11">
-        <v>69.900000000000006</v>
+        <v>79.984999999999999</v>
       </c>
       <c r="Z24" s="11">
-        <v>290.77</v>
+        <v>291.66000000000003</v>
       </c>
       <c r="AA24" s="11">
-        <v>1426.5</v>
+        <v>1479.6</v>
       </c>
       <c r="AB24" s="11">
-        <v>267814</v>
+        <v>141157</v>
       </c>
       <c r="AC24" s="11">
-        <v>77104</v>
+        <v>128547</v>
       </c>
       <c r="AD24" s="11">
-        <v>25649</v>
+        <v>23187</v>
       </c>
       <c r="AE24" s="11">
-        <v>1172</v>
+        <v>2470</v>
       </c>
       <c r="AF24" s="11">
-        <v>778.75</v>
+        <v>1049.166667</v>
       </c>
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A25" s="10">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="B25" s="11">
-        <v>2.1562540000000001</v>
+        <v>2.3418100000000002</v>
       </c>
       <c r="C25" s="11">
-        <v>74319.765438999995</v>
+        <v>71773.359093000006</v>
       </c>
       <c r="D25" s="11">
-        <v>1.0396719999999999</v>
+        <v>1.1343559999999999</v>
       </c>
       <c r="E25" s="11">
-        <v>15146.924349000001</v>
+        <v>16087.853573</v>
       </c>
       <c r="F25" s="11">
-        <v>6.04</v>
+        <v>9.51</v>
       </c>
       <c r="G25" s="11">
-        <v>67.099999999999994</v>
+        <v>65.400000000000006</v>
       </c>
       <c r="H25" s="11">
-        <v>10.57526</v>
+        <v>12.182824</v>
       </c>
       <c r="I25" s="11">
-        <v>174.76034200000001</v>
+        <v>169.996801</v>
       </c>
       <c r="J25" s="11">
-        <v>433.75</v>
+        <v>435.45</v>
       </c>
       <c r="K25" s="11">
-        <v>13.390751</v>
+        <v>13.874883000000001</v>
       </c>
       <c r="L25" s="11">
-        <v>13.349034</v>
+        <v>13.360428000000001</v>
       </c>
       <c r="M25" s="11">
-        <v>57595</v>
+        <v>57512</v>
       </c>
       <c r="N25" s="11">
-        <v>82114.5</v>
+        <v>61043</v>
       </c>
       <c r="O25" s="11">
-        <v>299594.5</v>
+        <v>296922</v>
       </c>
       <c r="P25" s="11">
-        <v>51376.5</v>
+        <v>48379</v>
       </c>
       <c r="Q25" s="20">
-        <v>3746.5</v>
+        <v>3978</v>
       </c>
       <c r="R25" s="20">
-        <v>23490.5</v>
+        <v>18874</v>
       </c>
       <c r="S25" s="20">
-        <v>75587</v>
+        <v>66383</v>
       </c>
       <c r="T25" s="20">
-        <v>12867.5</v>
+        <v>13135</v>
       </c>
       <c r="U25" s="20">
-        <v>53843.5</v>
+        <v>53530</v>
       </c>
       <c r="V25" s="20">
-        <v>58619.5</v>
+        <v>42170</v>
       </c>
       <c r="W25" s="20">
-        <v>223968.5</v>
+        <v>230492</v>
       </c>
       <c r="X25" s="20">
-        <v>38508</v>
+        <v>35245</v>
       </c>
       <c r="Y25" s="11">
-        <v>79.984999999999999</v>
+        <v>90.07</v>
       </c>
       <c r="Z25" s="11">
-        <v>291.66000000000003</v>
+        <v>294.2</v>
       </c>
       <c r="AA25" s="11">
-        <v>1479.6</v>
+        <v>1532.7</v>
       </c>
       <c r="AB25" s="11">
-        <v>141157</v>
+        <v>53530</v>
       </c>
       <c r="AC25" s="11">
-        <v>128547</v>
+        <v>54002</v>
       </c>
       <c r="AD25" s="11">
-        <v>23187</v>
+        <v>3709</v>
       </c>
       <c r="AE25" s="11">
-        <v>2470</v>
+        <v>2715</v>
       </c>
       <c r="AF25" s="11">
-        <v>1049.166667</v>
+        <v>1319.583333</v>
       </c>
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A26" s="10">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="B26" s="11">
-        <v>2.3418100000000002</v>
+        <v>2.6108530000000001</v>
       </c>
       <c r="C26" s="11">
-        <v>71773.359093000006</v>
+        <v>79056.336353000006</v>
       </c>
       <c r="D26" s="11">
-        <v>1.1343559999999999</v>
+        <v>0.87516799999999995</v>
       </c>
       <c r="E26" s="11">
-        <v>16087.853573</v>
+        <v>13748.624524000001</v>
       </c>
       <c r="F26" s="11">
-        <v>9.51</v>
+        <v>8.57</v>
       </c>
       <c r="G26" s="11">
-        <v>65.400000000000006</v>
+        <v>66.8</v>
       </c>
       <c r="H26" s="11">
-        <v>12.182824</v>
+        <v>10.656541000000001</v>
       </c>
       <c r="I26" s="11">
-        <v>169.996801</v>
+        <v>180.88040699999999</v>
       </c>
       <c r="J26" s="11">
-        <v>435.45</v>
+        <v>381.2</v>
       </c>
       <c r="K26" s="11">
-        <v>13.874883000000001</v>
+        <v>13.58709</v>
       </c>
       <c r="L26" s="11">
-        <v>13.360428000000001</v>
+        <v>13.345879999999999</v>
       </c>
       <c r="M26" s="11">
-        <v>57512</v>
+        <v>75864</v>
       </c>
       <c r="N26" s="11">
-        <v>61043</v>
+        <v>66226</v>
       </c>
       <c r="O26" s="11">
-        <v>296922</v>
+        <v>315229</v>
       </c>
       <c r="P26" s="11">
-        <v>48379</v>
+        <v>46555</v>
       </c>
       <c r="Q26" s="20">
-        <v>3978</v>
+        <v>14923</v>
       </c>
       <c r="R26" s="20">
-        <v>18874</v>
+        <v>22024</v>
       </c>
       <c r="S26" s="20">
-        <v>66383</v>
+        <v>84610</v>
       </c>
       <c r="T26" s="20">
-        <v>13135</v>
+        <v>12561</v>
       </c>
       <c r="U26" s="20">
-        <v>53530</v>
+        <v>60941</v>
       </c>
       <c r="V26" s="20">
-        <v>42170</v>
+        <v>44202</v>
       </c>
       <c r="W26" s="20">
-        <v>230492</v>
+        <v>230582</v>
       </c>
       <c r="X26" s="20">
-        <v>35245</v>
+        <v>33991</v>
       </c>
       <c r="Y26" s="11">
-        <v>90.07</v>
+        <v>88.3</v>
       </c>
       <c r="Z26" s="11">
-        <v>294.2</v>
+        <v>295.45999999999998</v>
       </c>
       <c r="AA26" s="11">
-        <v>1532.7</v>
+        <v>1585.8</v>
       </c>
       <c r="AB26" s="11">
-        <v>53530</v>
+        <v>97418</v>
       </c>
       <c r="AC26" s="11">
-        <v>54002</v>
+        <v>99007</v>
       </c>
       <c r="AD26" s="11">
-        <v>3709</v>
+        <v>18261</v>
       </c>
       <c r="AE26" s="11">
-        <v>2715</v>
+        <v>2670</v>
       </c>
       <c r="AF26" s="11">
-        <v>1319.583333</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A27" s="10">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="B27" s="11">
-        <v>2.6108530000000001</v>
+        <v>2.9270360000000002</v>
       </c>
       <c r="C27" s="11">
-        <v>79056.336353000006</v>
+        <v>109712.60879300001</v>
       </c>
       <c r="D27" s="11">
-        <v>0.87516799999999995</v>
+        <v>0.85815399999999997</v>
       </c>
       <c r="E27" s="11">
-        <v>13748.624524000001</v>
+        <v>15884.790272</v>
       </c>
       <c r="F27" s="11">
-        <v>8.57</v>
+        <v>12.08</v>
       </c>
       <c r="G27" s="11">
-        <v>66.8</v>
+        <v>66.7</v>
       </c>
       <c r="H27" s="11">
-        <v>10.656541000000001</v>
+        <v>10.377675</v>
       </c>
       <c r="I27" s="11">
-        <v>180.88040699999999</v>
+        <v>230.153685</v>
       </c>
       <c r="J27" s="11">
-        <v>381.2</v>
+        <v>367.2</v>
       </c>
       <c r="K27" s="11">
-        <v>13.58709</v>
+        <v>14.794839</v>
       </c>
       <c r="L27" s="11">
-        <v>13.345879999999999</v>
+        <v>13.535045</v>
       </c>
       <c r="M27" s="11">
-        <v>75864</v>
+        <v>66100</v>
       </c>
       <c r="N27" s="11">
-        <v>66226</v>
+        <v>65961</v>
       </c>
       <c r="O27" s="11">
-        <v>315229</v>
+        <v>315125</v>
       </c>
       <c r="P27" s="11">
-        <v>46555</v>
+        <v>31633</v>
       </c>
       <c r="Q27" s="20">
-        <v>14923</v>
+        <v>8567</v>
       </c>
       <c r="R27" s="20">
-        <v>22024</v>
+        <v>23315</v>
       </c>
       <c r="S27" s="20">
-        <v>84610</v>
+        <v>81915</v>
       </c>
       <c r="T27" s="20">
-        <v>12561</v>
+        <v>5708</v>
       </c>
       <c r="U27" s="20">
-        <v>60941</v>
+        <v>57532</v>
       </c>
       <c r="V27" s="20">
-        <v>44202</v>
+        <v>42646</v>
       </c>
       <c r="W27" s="20">
-        <v>230582</v>
+        <v>233175</v>
       </c>
       <c r="X27" s="20">
-        <v>33991</v>
+        <v>25925</v>
       </c>
       <c r="Y27" s="11">
-        <v>88.3</v>
+        <v>86.53</v>
       </c>
       <c r="Z27" s="11">
-        <v>295.45999999999998</v>
+        <v>295.69</v>
       </c>
       <c r="AA27" s="11">
-        <v>1585.8</v>
+        <v>1638.9</v>
       </c>
       <c r="AB27" s="11">
-        <v>97418</v>
+        <v>165872</v>
       </c>
       <c r="AC27" s="11">
-        <v>99007</v>
+        <v>143404</v>
       </c>
       <c r="AD27" s="11">
-        <v>18261</v>
+        <v>33772</v>
       </c>
       <c r="AE27" s="11">
-        <v>2670</v>
+        <v>2640</v>
       </c>
       <c r="AF27" s="11">
-        <v>1590</v>
+        <v>868</v>
       </c>
     </row>
     <row r="28" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A28" s="10">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="B28" s="11">
-        <v>2.9270360000000002</v>
+        <v>3.4030420000000001</v>
       </c>
       <c r="C28" s="11">
-        <v>109712.60879300001</v>
+        <v>105120.28866599999</v>
       </c>
       <c r="D28" s="11">
-        <v>0.85815399999999997</v>
+        <v>0.926311</v>
       </c>
       <c r="E28" s="11">
-        <v>15884.790272</v>
+        <v>19798.122179000002</v>
       </c>
       <c r="F28" s="11">
-        <v>12.08</v>
+        <v>9.34</v>
       </c>
       <c r="G28" s="11">
-        <v>66.7</v>
+        <v>67.400000000000006</v>
       </c>
       <c r="H28" s="11">
-        <v>10.377675</v>
+        <v>10.511326</v>
       </c>
       <c r="I28" s="11">
-        <v>230.153685</v>
+        <v>247.878015</v>
       </c>
       <c r="J28" s="11">
-        <v>367.2</v>
+        <v>301.05</v>
       </c>
       <c r="K28" s="11">
-        <v>14.794839</v>
+        <v>14.991778999999999</v>
       </c>
       <c r="L28" s="11">
-        <v>13.535045</v>
+        <v>13.715916999999999</v>
       </c>
       <c r="M28" s="11">
-        <v>66100</v>
+        <v>71062</v>
       </c>
       <c r="N28" s="11">
-        <v>65961</v>
+        <v>67601</v>
       </c>
       <c r="O28" s="11">
-        <v>315125</v>
+        <v>310120</v>
       </c>
       <c r="P28" s="11">
-        <v>31633</v>
+        <v>37508</v>
       </c>
       <c r="Q28" s="20">
-        <v>8567</v>
+        <v>10622</v>
       </c>
       <c r="R28" s="20">
-        <v>23315</v>
+        <v>21803</v>
       </c>
       <c r="S28" s="20">
-        <v>81915</v>
+        <v>80456</v>
       </c>
       <c r="T28" s="20">
-        <v>5708</v>
+        <v>9742</v>
       </c>
       <c r="U28" s="20">
-        <v>57532</v>
+        <v>60440</v>
       </c>
       <c r="V28" s="20">
-        <v>42646</v>
+        <v>45798</v>
       </c>
       <c r="W28" s="20">
-        <v>233175</v>
+        <v>229629</v>
       </c>
       <c r="X28" s="20">
-        <v>25925</v>
+        <v>27766</v>
       </c>
       <c r="Y28" s="11">
-        <v>86.53</v>
+        <v>68.59</v>
       </c>
       <c r="Z28" s="11">
-        <v>295.69</v>
+        <v>295.42</v>
       </c>
       <c r="AA28" s="11">
-        <v>1638.9</v>
+        <v>1692</v>
       </c>
       <c r="AB28" s="11">
-        <v>165872</v>
+        <v>216309</v>
       </c>
       <c r="AC28" s="11">
-        <v>143404</v>
+        <v>175199</v>
       </c>
       <c r="AD28" s="11">
-        <v>33772</v>
+        <v>43787</v>
       </c>
       <c r="AE28" s="11">
-        <v>2640</v>
+        <v>1629</v>
       </c>
       <c r="AF28" s="11">
-        <v>868</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="29" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B29" s="11">
-        <v>3.4030420000000001</v>
+        <v>2.9975749999999999</v>
       </c>
       <c r="C29" s="11">
-        <v>105120.28866599999</v>
+        <v>110963.315862</v>
       </c>
       <c r="D29" s="11">
-        <v>0.926311</v>
+        <v>0.92500300000000002</v>
       </c>
       <c r="E29" s="11">
-        <v>19798.122179000002</v>
+        <v>17360.471361</v>
       </c>
       <c r="F29" s="11">
-        <v>9.34</v>
+        <v>10.09</v>
       </c>
       <c r="G29" s="11">
-        <v>67.400000000000006</v>
+        <v>68.5</v>
       </c>
       <c r="H29" s="11">
-        <v>10.511326</v>
+        <v>9.6488479999999992</v>
       </c>
       <c r="I29" s="11">
-        <v>247.878015</v>
+        <v>239.42585700000001</v>
       </c>
       <c r="J29" s="11">
-        <v>301.05</v>
+        <v>285.2</v>
       </c>
       <c r="K29" s="11">
-        <v>14.991778999999999</v>
+        <v>14.833494999999999</v>
       </c>
       <c r="L29" s="11">
-        <v>13.715916999999999</v>
+        <v>14.174294</v>
       </c>
       <c r="M29" s="11">
-        <v>71062</v>
+        <v>73610</v>
       </c>
       <c r="N29" s="11">
-        <v>67601</v>
+        <v>75812</v>
       </c>
       <c r="O29" s="11">
-        <v>310120</v>
+        <v>304865</v>
       </c>
       <c r="P29" s="11">
-        <v>37508</v>
+        <v>38253</v>
       </c>
       <c r="Q29" s="20">
-        <v>10622</v>
+        <v>9712</v>
       </c>
       <c r="R29" s="20">
-        <v>21803</v>
+        <v>27588</v>
       </c>
       <c r="S29" s="20">
-        <v>80456</v>
+        <v>80726</v>
       </c>
       <c r="T29" s="20">
-        <v>9742</v>
+        <v>10562</v>
       </c>
       <c r="U29" s="20">
-        <v>60440</v>
+        <v>63897</v>
       </c>
       <c r="V29" s="20">
-        <v>45798</v>
+        <v>48222</v>
       </c>
       <c r="W29" s="20">
-        <v>229629</v>
+        <v>224114</v>
       </c>
       <c r="X29" s="20">
-        <v>27766</v>
+        <v>27690</v>
       </c>
       <c r="Y29" s="11">
-        <v>68.59</v>
+        <v>77.819999999999993</v>
       </c>
       <c r="Z29" s="11">
-        <v>295.42</v>
+        <v>294.7</v>
       </c>
       <c r="AA29" s="11">
-        <v>1692</v>
+        <v>1745.1</v>
       </c>
       <c r="AB29" s="11">
-        <v>216309</v>
+        <v>249919</v>
       </c>
       <c r="AC29" s="11">
-        <v>175199</v>
+        <v>259510</v>
       </c>
       <c r="AD29" s="11">
-        <v>43787</v>
+        <v>54506</v>
       </c>
       <c r="AE29" s="11">
-        <v>1629</v>
+        <v>777</v>
       </c>
       <c r="AF29" s="11">
-        <v>1545</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A30" s="10">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B30" s="11">
-        <v>2.9975749999999999</v>
+        <v>2.210331</v>
       </c>
       <c r="C30" s="11">
-        <v>110963.315862</v>
+        <v>107441.247456</v>
       </c>
       <c r="D30" s="11">
-        <v>0.92500300000000002</v>
+        <v>0.90799399999999997</v>
       </c>
       <c r="E30" s="11">
-        <v>17360.471361</v>
+        <v>16790.507846</v>
       </c>
       <c r="F30" s="11">
-        <v>10.09</v>
+        <v>8.3699999999999992</v>
       </c>
       <c r="G30" s="11">
-        <v>68.5</v>
+        <v>68.099999999999994</v>
       </c>
       <c r="H30" s="11">
-        <v>9.6488479999999992</v>
+        <v>10.423719</v>
       </c>
       <c r="I30" s="11">
-        <v>239.42585700000001</v>
+        <v>225.54091</v>
       </c>
       <c r="J30" s="11">
-        <v>285.2</v>
+        <v>306.39999999999998</v>
       </c>
       <c r="K30" s="11">
-        <v>14.833494999999999</v>
+        <v>15.120673</v>
       </c>
       <c r="L30" s="11">
-        <v>14.174294</v>
+        <v>14.916763</v>
       </c>
       <c r="M30" s="11">
-        <v>73610</v>
+        <v>72322</v>
       </c>
       <c r="N30" s="11">
-        <v>75812</v>
+        <v>85275</v>
       </c>
       <c r="O30" s="11">
-        <v>304865</v>
+        <v>315151</v>
       </c>
       <c r="P30" s="11">
-        <v>38253</v>
+        <v>38533</v>
       </c>
       <c r="Q30" s="20">
-        <v>9712</v>
+        <v>6898</v>
       </c>
       <c r="R30" s="20">
-        <v>27588</v>
+        <v>28511</v>
       </c>
       <c r="S30" s="20">
-        <v>80726</v>
+        <v>83804</v>
       </c>
       <c r="T30" s="20">
-        <v>10562</v>
+        <v>9917</v>
       </c>
       <c r="U30" s="20">
-        <v>63897</v>
+        <v>65423</v>
       </c>
       <c r="V30" s="20">
-        <v>48222</v>
+        <v>56764</v>
       </c>
       <c r="W30" s="20">
-        <v>224114</v>
+        <v>231309</v>
       </c>
       <c r="X30" s="20">
-        <v>27690</v>
+        <v>28611</v>
       </c>
       <c r="Y30" s="11">
-        <v>77.819999999999993</v>
+        <v>93.51</v>
       </c>
       <c r="Z30" s="11">
-        <v>294.7</v>
+        <v>294.32</v>
       </c>
       <c r="AA30" s="11">
-        <v>1745.1</v>
+        <v>1798.2</v>
       </c>
       <c r="AB30" s="11">
-        <v>249919</v>
+        <v>279211</v>
       </c>
       <c r="AC30" s="11">
-        <v>259510</v>
+        <v>127487</v>
       </c>
       <c r="AD30" s="11">
-        <v>54506</v>
+        <v>37735</v>
       </c>
       <c r="AE30" s="11">
-        <v>777</v>
+        <v>648</v>
       </c>
       <c r="AF30" s="11">
-        <v>248</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A31" s="10">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B31" s="11">
-        <v>2.210331</v>
+        <v>2.2697189999999998</v>
       </c>
       <c r="C31" s="11">
-        <v>107441.247456</v>
+        <v>96475.806196999998</v>
       </c>
       <c r="D31" s="11">
-        <v>0.90799399999999997</v>
+        <v>0.76849699999999999</v>
       </c>
       <c r="E31" s="11">
-        <v>16790.507846</v>
+        <v>15425.082779</v>
       </c>
       <c r="F31" s="11">
-        <v>8.3699999999999992</v>
+        <v>8.08</v>
       </c>
       <c r="G31" s="11">
-        <v>68.099999999999994</v>
+        <v>67.099999999999994</v>
       </c>
       <c r="H31" s="11">
-        <v>10.423719</v>
+        <v>10.608466999999999</v>
       </c>
       <c r="I31" s="11">
-        <v>225.54091</v>
+        <v>186.34489099999999</v>
       </c>
       <c r="J31" s="11">
-        <v>306.39999999999998</v>
+        <v>315.2</v>
       </c>
       <c r="K31" s="11">
-        <v>15.120673</v>
+        <v>15.172575</v>
       </c>
       <c r="L31" s="11">
-        <v>14.916763</v>
+        <v>28.785724999999999</v>
       </c>
       <c r="M31" s="11">
-        <v>72322</v>
+        <v>83214</v>
       </c>
       <c r="N31" s="11">
-        <v>85275</v>
+        <v>50152</v>
       </c>
       <c r="O31" s="11">
-        <v>315151</v>
+        <v>321688</v>
       </c>
       <c r="P31" s="11">
-        <v>38533</v>
+        <v>28817</v>
       </c>
       <c r="Q31" s="20">
-        <v>6898</v>
+        <v>9991</v>
       </c>
       <c r="R31" s="20">
-        <v>28511</v>
+        <v>18704</v>
       </c>
       <c r="S31" s="20">
-        <v>83804</v>
+        <v>73581</v>
       </c>
       <c r="T31" s="20">
-        <v>9917</v>
+        <v>7839</v>
       </c>
       <c r="U31" s="20">
-        <v>65423</v>
+        <v>73223</v>
       </c>
       <c r="V31" s="20">
-        <v>56764</v>
+        <v>31449</v>
       </c>
       <c r="W31" s="20">
-        <v>231309</v>
+        <v>248093</v>
       </c>
       <c r="X31" s="20">
-        <v>28611</v>
+        <v>20977</v>
       </c>
       <c r="Y31" s="11">
-        <v>93.51</v>
+        <v>76.17</v>
       </c>
       <c r="Z31" s="11">
-        <v>294.32</v>
+        <v>296.24</v>
       </c>
       <c r="AA31" s="11">
-        <v>1798.2</v>
+        <v>1851.3</v>
       </c>
       <c r="AB31" s="11">
-        <v>279211</v>
+        <v>155800</v>
       </c>
       <c r="AC31" s="11">
-        <v>127487</v>
+        <v>191462</v>
       </c>
       <c r="AD31" s="11">
-        <v>37735</v>
+        <v>39935</v>
       </c>
       <c r="AE31" s="11">
-        <v>648</v>
+        <v>468</v>
       </c>
       <c r="AF31" s="11">
-        <v>1302</v>
+        <v>604</v>
       </c>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A32" s="10">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B32" s="11">
-        <v>2.2697189999999998</v>
+        <v>1.7425330000000001</v>
       </c>
       <c r="C32" s="11">
-        <v>96475.806196999998</v>
+        <v>92044.926760000002</v>
       </c>
       <c r="D32" s="11">
-        <v>0.76849699999999999</v>
+        <v>0.839584</v>
       </c>
       <c r="E32" s="11">
-        <v>15425.082779</v>
+        <v>16818.249621999999</v>
       </c>
       <c r="F32" s="11">
-        <v>8.08</v>
+        <v>5.84</v>
       </c>
       <c r="G32" s="11">
-        <v>67.099999999999994</v>
+        <v>68.3</v>
       </c>
       <c r="H32" s="11">
-        <v>10.608466999999999</v>
+        <v>10.479568</v>
       </c>
       <c r="I32" s="11">
-        <v>186.34489099999999</v>
+        <v>210.46378899999999</v>
       </c>
       <c r="J32" s="11">
-        <v>315.2</v>
+        <v>283.89999999999998</v>
       </c>
       <c r="K32" s="11">
-        <v>15.172575</v>
+        <v>15.463456000000001</v>
       </c>
       <c r="L32" s="11">
-        <v>28.785724999999999</v>
+        <v>29.231781999999999</v>
       </c>
       <c r="M32" s="11">
-        <v>83214</v>
+        <v>90880</v>
       </c>
       <c r="N32" s="11">
-        <v>50152</v>
+        <v>74128</v>
       </c>
       <c r="O32" s="11">
-        <v>321688</v>
+        <v>327300</v>
       </c>
       <c r="P32" s="11">
-        <v>28817</v>
+        <v>29146</v>
       </c>
       <c r="Q32" s="20">
-        <v>9991</v>
+        <v>14196</v>
       </c>
       <c r="R32" s="20">
-        <v>18704</v>
+        <v>24767</v>
       </c>
       <c r="S32" s="20">
-        <v>73581</v>
+        <v>83138</v>
       </c>
       <c r="T32" s="20">
-        <v>7839</v>
+        <v>7103</v>
       </c>
       <c r="U32" s="20">
-        <v>73223</v>
+        <v>76683</v>
       </c>
       <c r="V32" s="20">
-        <v>31449</v>
+        <v>49357</v>
       </c>
       <c r="W32" s="20">
-        <v>248093</v>
+        <v>244143</v>
       </c>
       <c r="X32" s="20">
-        <v>20977</v>
+        <v>22044</v>
       </c>
       <c r="Y32" s="11">
-        <v>76.17</v>
+        <v>76.11</v>
       </c>
       <c r="Z32" s="11">
-        <v>296.24</v>
+        <v>295.93</v>
       </c>
       <c r="AA32" s="11">
-        <v>1851.3</v>
+        <v>1904.4</v>
       </c>
       <c r="AB32" s="11">
-        <v>155800</v>
+        <v>268582</v>
       </c>
       <c r="AC32" s="11">
-        <v>191462</v>
+        <v>198314</v>
       </c>
       <c r="AD32" s="11">
-        <v>39935</v>
+        <v>43968</v>
       </c>
       <c r="AE32" s="11">
-        <v>468</v>
+        <v>626</v>
       </c>
       <c r="AF32" s="11">
-        <v>604</v>
+        <v>932</v>
       </c>
     </row>
     <row r="33" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A33" s="10">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B33" s="11">
-        <v>1.7425330000000001</v>
+        <v>2.5139230000000001</v>
       </c>
       <c r="C33" s="11">
-        <v>92044.926760000002</v>
+        <v>107642.621608</v>
       </c>
       <c r="D33" s="11">
-        <v>0.839584</v>
+        <v>1.102169</v>
       </c>
       <c r="E33" s="11">
-        <v>16818.249621999999</v>
+        <v>21804.002927000001</v>
       </c>
       <c r="F33" s="11">
-        <v>5.84</v>
+        <v>12.03</v>
       </c>
       <c r="G33" s="11">
-        <v>68.3</v>
+        <v>66.900000000000006</v>
       </c>
       <c r="H33" s="11">
-        <v>10.479568</v>
+        <v>12.802387</v>
       </c>
       <c r="I33" s="11">
-        <v>210.46378899999999</v>
+        <v>199.133115</v>
       </c>
       <c r="J33" s="11">
-        <v>283.89999999999998</v>
+        <v>409.54</v>
       </c>
       <c r="K33" s="11">
-        <v>15.463456000000001</v>
+        <v>16.061176</v>
       </c>
       <c r="L33" s="11">
-        <v>29.231781999999999</v>
+        <v>31.806149000000001</v>
       </c>
       <c r="M33" s="11">
-        <v>90880</v>
+        <v>85817</v>
       </c>
       <c r="N33" s="11">
-        <v>74128</v>
+        <v>40110</v>
       </c>
       <c r="O33" s="11">
-        <v>327300</v>
+        <v>363667</v>
       </c>
       <c r="P33" s="11">
-        <v>29146</v>
+        <v>36637</v>
       </c>
       <c r="Q33" s="20">
-        <v>14196</v>
+        <v>11326</v>
       </c>
       <c r="R33" s="20">
-        <v>24767</v>
+        <v>11916</v>
       </c>
       <c r="S33" s="20">
-        <v>83138</v>
+        <v>88210</v>
       </c>
       <c r="T33" s="20">
-        <v>7103</v>
+        <v>10432</v>
       </c>
       <c r="U33" s="20">
-        <v>76683</v>
+        <v>74487</v>
       </c>
       <c r="V33" s="20">
-        <v>49357</v>
+        <v>28193</v>
       </c>
       <c r="W33" s="20">
-        <v>244143</v>
+        <v>275427</v>
       </c>
       <c r="X33" s="20">
-        <v>22044</v>
+        <v>26203</v>
       </c>
       <c r="Y33" s="11">
-        <v>76.11</v>
+        <v>91.33</v>
       </c>
       <c r="Z33" s="11">
-        <v>295.93</v>
+        <v>298.45</v>
       </c>
       <c r="AA33" s="11">
-        <v>1904.4</v>
+        <v>1957.5</v>
       </c>
       <c r="AB33" s="11">
-        <v>268582</v>
+        <v>120659</v>
       </c>
       <c r="AC33" s="11">
-        <v>198314</v>
+        <v>57704</v>
       </c>
       <c r="AD33" s="11">
-        <v>43968</v>
+        <v>12145</v>
       </c>
       <c r="AE33" s="11">
-        <v>626</v>
+        <v>2180</v>
       </c>
       <c r="AF33" s="11">
-        <v>932</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="34" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A34" s="10">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B34" s="11">
-        <v>2.5139230000000001</v>
+        <v>1.939756</v>
       </c>
       <c r="C34" s="11">
-        <v>107642.621608</v>
+        <v>80821.071186000001</v>
       </c>
       <c r="D34" s="11">
-        <v>1.102169</v>
+        <v>0.960179</v>
       </c>
       <c r="E34" s="11">
-        <v>21804.002927000001</v>
+        <v>17695.211750999999</v>
       </c>
       <c r="F34" s="11">
-        <v>12.03</v>
+        <v>8.92</v>
       </c>
       <c r="G34" s="11">
-        <v>66.900000000000006</v>
+        <v>66.400000000000006</v>
       </c>
       <c r="H34" s="11">
-        <v>12.802387</v>
+        <v>11.854062000000001</v>
       </c>
       <c r="I34" s="11">
-        <v>199.133115</v>
+        <v>184.55339699999999</v>
       </c>
       <c r="J34" s="11">
-        <v>409.54</v>
+        <v>667.17</v>
       </c>
       <c r="K34" s="11">
-        <v>16.061176</v>
+        <v>15.453386</v>
       </c>
       <c r="L34" s="11">
-        <v>31.806149000000001</v>
+        <v>35.963047000000003</v>
       </c>
       <c r="M34" s="11">
-        <v>85817</v>
+        <v>84566</v>
       </c>
       <c r="N34" s="11">
-        <v>40110</v>
+        <v>50811</v>
       </c>
       <c r="O34" s="11">
-        <v>363667</v>
+        <v>361525</v>
       </c>
       <c r="P34" s="11">
-        <v>36637</v>
+        <v>42023</v>
       </c>
       <c r="Q34" s="20">
-        <v>11326</v>
+        <v>8101</v>
       </c>
       <c r="R34" s="20">
-        <v>11916</v>
+        <v>16715</v>
       </c>
       <c r="S34" s="20">
-        <v>88210</v>
+        <v>91551</v>
       </c>
       <c r="T34" s="20">
-        <v>10432</v>
+        <v>16233</v>
       </c>
       <c r="U34" s="20">
-        <v>74487</v>
+        <v>76465</v>
       </c>
       <c r="V34" s="20">
-        <v>28193</v>
+        <v>34096</v>
       </c>
       <c r="W34" s="20">
-        <v>275427</v>
+        <v>269909</v>
       </c>
       <c r="X34" s="20">
-        <v>26203</v>
+        <v>25790</v>
       </c>
       <c r="Y34" s="11">
-        <v>91.33</v>
+        <v>94.85</v>
       </c>
       <c r="Z34" s="11">
-        <v>298.45</v>
+        <v>299.43</v>
       </c>
       <c r="AA34" s="11">
-        <v>1957.5</v>
+        <v>2010.6</v>
       </c>
       <c r="AB34" s="11">
-        <v>120659</v>
+        <v>111483</v>
       </c>
       <c r="AC34" s="11">
-        <v>57704</v>
+        <v>82339</v>
       </c>
       <c r="AD34" s="11">
-        <v>12145</v>
+        <v>14843</v>
       </c>
       <c r="AE34" s="11">
-        <v>2180</v>
+        <v>2645</v>
       </c>
       <c r="AF34" s="11">
-        <v>1440</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="35" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A35" s="10">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B35" s="11">
-        <v>1.939756</v>
+        <v>1.7387999999999999</v>
       </c>
       <c r="C35" s="11">
-        <v>80821.071186000001</v>
+        <v>69963.013120000003</v>
       </c>
       <c r="D35" s="11">
-        <v>0.960179</v>
+        <v>0.80419499999999999</v>
       </c>
       <c r="E35" s="11">
-        <v>17695.211750999999</v>
+        <v>16725.250080000002</v>
       </c>
       <c r="F35" s="11">
-        <v>8.92</v>
+        <v>4.34</v>
       </c>
       <c r="G35" s="11">
-        <v>66.400000000000006</v>
+        <v>69.099999999999994</v>
       </c>
       <c r="H35" s="11">
-        <v>11.854062000000001</v>
+        <v>12.42</v>
       </c>
       <c r="I35" s="11">
-        <v>184.55339699999999</v>
+        <v>174.88239999999999</v>
       </c>
       <c r="J35" s="11">
-        <v>667.17</v>
+        <v>413.32</v>
       </c>
       <c r="K35" s="11">
-        <v>15.453386</v>
+        <v>16.311599999999999</v>
       </c>
       <c r="L35" s="11">
-        <v>35.963047000000003</v>
+        <v>40.894469000000001</v>
       </c>
       <c r="M35" s="11">
-        <v>84566</v>
+        <v>87937</v>
       </c>
       <c r="N35" s="11">
-        <v>50811</v>
+        <v>49774</v>
       </c>
       <c r="O35" s="11">
-        <v>361525</v>
+        <v>376870</v>
       </c>
       <c r="P35" s="11">
-        <v>42023</v>
-      </c>
-      <c r="Q35" s="20">
-        <v>8101</v>
-      </c>
-      <c r="R35" s="20">
-        <v>16715</v>
-      </c>
-      <c r="S35" s="20">
-        <v>91551</v>
-      </c>
-      <c r="T35" s="20">
-        <v>16233</v>
-      </c>
-      <c r="U35" s="20">
-        <v>76465</v>
-      </c>
-      <c r="V35" s="20">
-        <v>34096</v>
-      </c>
-      <c r="W35" s="20">
-        <v>269909</v>
-      </c>
-      <c r="X35" s="20">
-        <v>25790</v>
+        <v>35989</v>
+      </c>
+      <c r="Q35" s="21">
+        <v>12690</v>
+      </c>
+      <c r="R35" s="21">
+        <v>17092</v>
+      </c>
+      <c r="S35" s="21">
+        <v>98742</v>
+      </c>
+      <c r="T35" s="21">
+        <v>10606</v>
+      </c>
+      <c r="U35" s="21">
+        <v>75243</v>
+      </c>
+      <c r="V35" s="21">
+        <v>32677</v>
+      </c>
+      <c r="W35" s="21">
+        <v>277830</v>
+      </c>
+      <c r="X35" s="21">
+        <v>25366</v>
       </c>
       <c r="Y35" s="11">
-        <v>94.85</v>
+        <v>85.81</v>
       </c>
       <c r="Z35" s="11">
-        <v>299.43</v>
+        <v>299.56</v>
       </c>
       <c r="AA35" s="11">
-        <v>2010.6</v>
+        <v>2063.6999999999998</v>
       </c>
       <c r="AB35" s="11">
-        <v>111483</v>
+        <v>225495</v>
       </c>
       <c r="AC35" s="11">
-        <v>82339</v>
+        <v>189551</v>
       </c>
       <c r="AD35" s="11">
-        <v>14843</v>
+        <v>46119</v>
       </c>
       <c r="AE35" s="11">
-        <v>2645</v>
+        <v>2265</v>
       </c>
       <c r="AF35" s="11">
-        <v>1580</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="36" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A36" s="10">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B36" s="11">
-        <v>1.7387999999999999</v>
+        <v>1.7969999999999999</v>
       </c>
       <c r="C36" s="11">
-        <v>69963.013120000003</v>
+        <v>71151.604000000007</v>
       </c>
       <c r="D36" s="11">
-        <v>0.80419499999999999</v>
+        <v>0.93840000000000001</v>
       </c>
       <c r="E36" s="11">
-        <v>16725.250080000002</v>
+        <v>18370.973000000002</v>
       </c>
       <c r="F36" s="11">
-        <v>4.34</v>
+        <v>4.01</v>
       </c>
       <c r="G36" s="11">
-        <v>69.099999999999994</v>
+        <v>72.8</v>
       </c>
       <c r="H36" s="11">
-        <v>12.42</v>
+        <v>13</v>
       </c>
       <c r="I36" s="11">
-        <v>174.88239999999999</v>
+        <v>176.6</v>
       </c>
       <c r="J36" s="11">
-        <v>413.32</v>
+        <v>386.33</v>
       </c>
       <c r="K36" s="11">
-        <v>16.311599999999999</v>
+        <v>16.11</v>
       </c>
       <c r="L36" s="11">
-        <v>40.894469000000001</v>
+        <v>46.861249999999998</v>
       </c>
       <c r="M36" s="11">
-        <v>87937</v>
+        <v>87422.399999999994</v>
       </c>
       <c r="N36" s="11">
-        <v>49774</v>
+        <v>45773.1</v>
       </c>
       <c r="O36" s="11">
-        <v>376870</v>
+        <v>393586.7</v>
       </c>
       <c r="P36" s="11">
-        <v>35989</v>
+        <v>42688.7</v>
       </c>
       <c r="Q36" s="21">
-        <v>12690</v>
+        <v>2526</v>
       </c>
       <c r="R36" s="21">
-        <v>17092</v>
+        <v>19126</v>
       </c>
       <c r="S36" s="21">
-        <v>98742</v>
+        <v>83371</v>
       </c>
       <c r="T36" s="21">
-        <v>10606</v>
+        <v>15057</v>
       </c>
       <c r="U36" s="21">
-        <v>75243</v>
+        <v>66590</v>
       </c>
       <c r="V36" s="21">
-        <v>32677</v>
+        <v>35632</v>
       </c>
       <c r="W36" s="21">
-        <v>277830</v>
+        <v>238688</v>
       </c>
       <c r="X36" s="21">
-        <v>25366</v>
+        <v>24865</v>
       </c>
       <c r="Y36" s="11">
-        <v>85.81</v>
+        <v>96.26</v>
       </c>
       <c r="Z36" s="11">
-        <v>299.56</v>
+        <v>297.64</v>
       </c>
       <c r="AA36" s="11">
-        <v>2063.6999999999998</v>
+        <v>2116.8000000000002</v>
       </c>
       <c r="AB36" s="11">
-        <v>225495</v>
+        <v>171091.1</v>
       </c>
       <c r="AC36" s="11">
-        <v>189551</v>
+        <v>107934.9</v>
       </c>
       <c r="AD36" s="11">
-        <v>46119</v>
+        <v>26374.9</v>
       </c>
       <c r="AE36" s="11">
-        <v>2265</v>
+        <v>3320.7</v>
       </c>
       <c r="AF36" s="11">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="37" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A37" s="10">
-        <v>2024</v>
-      </c>
-      <c r="B37" s="11">
-        <v>1.7969999999999999</v>
-      </c>
-      <c r="C37" s="11">
-        <v>71151.604000000007</v>
-      </c>
-      <c r="D37" s="11">
-        <v>0.93840000000000001</v>
-      </c>
-      <c r="E37" s="11">
-        <v>18370.973000000002</v>
-      </c>
-      <c r="F37" s="11">
-        <v>4.01</v>
-      </c>
-      <c r="G37" s="11">
-        <v>72.8</v>
-      </c>
-      <c r="H37" s="11">
-        <v>13</v>
-      </c>
-      <c r="I37" s="11">
-        <v>176.6</v>
-      </c>
-      <c r="J37" s="11">
-        <v>386.33</v>
-      </c>
-      <c r="K37" s="11">
-        <v>16.11</v>
-      </c>
-      <c r="L37" s="11">
-        <v>46.861249999999998</v>
-      </c>
-      <c r="M37" s="11">
-        <v>87422.399999999994</v>
-      </c>
-      <c r="N37" s="11">
-        <v>45773.1</v>
-      </c>
-      <c r="O37" s="11">
-        <v>393586.7</v>
-      </c>
-      <c r="P37" s="11">
-        <v>42688.7</v>
-      </c>
-      <c r="Q37" s="21">
-        <v>2526</v>
-      </c>
-      <c r="R37" s="21">
-        <v>19126</v>
-      </c>
-      <c r="S37" s="21">
-        <v>83371</v>
-      </c>
-      <c r="T37" s="21">
-        <v>15057</v>
-      </c>
-      <c r="U37" s="21">
-        <v>66590</v>
-      </c>
-      <c r="V37" s="21">
-        <v>35632</v>
-      </c>
-      <c r="W37" s="21">
-        <v>238688</v>
-      </c>
-      <c r="X37" s="21">
-        <v>24865</v>
-      </c>
-      <c r="Y37" s="11">
-        <v>96.26</v>
-      </c>
-      <c r="Z37" s="11">
-        <v>297.64</v>
-      </c>
-      <c r="AA37" s="11">
-        <v>2116.8000000000002</v>
-      </c>
-      <c r="AB37" s="11">
-        <v>171091.1</v>
-      </c>
-      <c r="AC37" s="11">
-        <v>107934.9</v>
-      </c>
-      <c r="AD37" s="11">
-        <v>26374.9</v>
-      </c>
-      <c r="AE37" s="11">
-        <v>3320.7</v>
-      </c>
-      <c r="AF37" s="11">
         <v>2183.1999999999998</v>
       </c>
     </row>
@@ -21821,15 +21723,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C0C065D4DE56964884282D8F503EB12D" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cfa0f9876d3650d261453c6251028662">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="26585f66-47fc-498d-b213-b46953568bdc" xmlns:ns3="984dc5cf-9f96-4254-8c6c-2d4fc144aaf2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="61f3943096767e2b3d869813e253bb59" ns2:_="" ns3:_="">
     <xsd:import namespace="26585f66-47fc-498d-b213-b46953568bdc"/>
@@ -22040,6 +21933,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -22051,14 +21953,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BCB75A9-047C-49FD-97F3-E954E4582F73}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0E3D96E-C286-4914-9D33-19BF1F42696C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22077,6 +21971,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BCB75A9-047C-49FD-97F3-E954E4582F73}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58DF89A4-C330-4DFA-9A84-C3DE3B38B451}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Changed name to Groundwater
</commit_message>
<xml_diff>
--- a/FinalDataset.xlsx
+++ b/FinalDataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/krishnaprasadpa/Desktop/Part time/aimm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rneribar/AIMM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EBD4DBD-4DAB-2842-8A66-5DCAE2477367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0063FCE4-D74B-7847-AE76-97B309D0608C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="760" windowWidth="29060" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1180" yWindow="760" windowWidth="29060" windowHeight="17780" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.Original" sheetId="28" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="102">
   <si>
     <t>Year</t>
   </si>
@@ -341,6 +341,12 @@
   </si>
   <si>
     <t>SW TDS (Hueco)</t>
+  </si>
+  <si>
+    <t>Groundwater  level (Mesilla)</t>
+  </si>
+  <si>
+    <t>Groundwater  level (Hueco)</t>
   </si>
 </sst>
 </file>
@@ -7574,7 +7580,9 @@
     <col min="1" max="1" width="10.83203125" style="5"/>
     <col min="2" max="16" width="10.83203125" style="1"/>
     <col min="17" max="24" width="10.83203125" style="21"/>
-    <col min="25" max="16384" width="10.83203125" style="1"/>
+    <col min="25" max="25" width="11.5" style="1" customWidth="1"/>
+    <col min="26" max="26" width="11.33203125" style="1" customWidth="1"/>
+    <col min="27" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" s="9" customFormat="1" ht="64" x14ac:dyDescent="0.2">
@@ -7847,10 +7855,10 @@
         <v>23</v>
       </c>
       <c r="Y3" s="22" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="Z3" s="22" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="AA3" s="22" t="s">
         <v>97</v>
@@ -7974,127 +7982,127 @@
         <v>46</v>
       </c>
       <c r="B5" s="9">
-        <f>MAX(B6:B36)</f>
+        <f t="shared" ref="B5:AF5" si="0">MAX(B6:B36)</f>
         <v>3.4064709999999998</v>
       </c>
       <c r="C5" s="9">
-        <f>MAX(C6:C36)</f>
+        <f t="shared" si="0"/>
         <v>154688.542193</v>
       </c>
       <c r="D5" s="9">
-        <f>MAX(D6:D36)</f>
+        <f t="shared" si="0"/>
         <v>1.583216</v>
       </c>
       <c r="E5" s="9">
-        <f>MAX(E6:E36)</f>
+        <f t="shared" si="0"/>
         <v>28180.264358</v>
       </c>
       <c r="F5" s="9">
-        <f>MAX(F6:F36)</f>
+        <f t="shared" si="0"/>
         <v>17.510000000000002</v>
       </c>
       <c r="G5" s="9">
-        <f>MAX(G6:G36)</f>
+        <f t="shared" si="0"/>
         <v>72.8</v>
       </c>
       <c r="H5" s="9">
-        <f>MAX(H6:H36)</f>
+        <f t="shared" si="0"/>
         <v>15.456422</v>
       </c>
       <c r="I5" s="9">
-        <f>MAX(I6:I36)</f>
+        <f t="shared" si="0"/>
         <v>611.711996</v>
       </c>
       <c r="J5" s="9">
-        <f>MAX(J6:J36)</f>
+        <f t="shared" si="0"/>
         <v>667.17</v>
       </c>
       <c r="K5" s="9">
-        <f>MAX(K6:K36)</f>
+        <f t="shared" si="0"/>
         <v>16.311599999999999</v>
       </c>
       <c r="L5" s="9">
-        <f>MAX(L6:L36)</f>
+        <f t="shared" si="0"/>
         <v>46.861249999999998</v>
       </c>
       <c r="M5" s="9">
-        <f>MAX(M6:M36)</f>
+        <f t="shared" si="0"/>
         <v>90880</v>
       </c>
       <c r="N5" s="9">
-        <f>MAX(N6:N36)</f>
+        <f t="shared" si="0"/>
         <v>125650</v>
       </c>
       <c r="O5" s="9">
-        <f>MAX(O6:O36)</f>
+        <f t="shared" si="0"/>
         <v>393586.7</v>
       </c>
       <c r="P5" s="9">
-        <f>MAX(P6:P36)</f>
+        <f t="shared" si="0"/>
         <v>91721</v>
       </c>
       <c r="Q5" s="19">
-        <f>MAX(Q6:Q36)</f>
+        <f t="shared" si="0"/>
         <v>14923</v>
       </c>
       <c r="R5" s="19">
-        <f>MAX(R6:R36)</f>
+        <f t="shared" si="0"/>
         <v>40932</v>
       </c>
       <c r="S5" s="19">
-        <f>MAX(S6:S36)</f>
+        <f t="shared" si="0"/>
         <v>98742</v>
       </c>
       <c r="T5" s="19">
-        <f>MAX(T6:T36)</f>
+        <f t="shared" si="0"/>
         <v>25761</v>
       </c>
       <c r="U5" s="19">
-        <f>MAX(U6:U36)</f>
+        <f t="shared" si="0"/>
         <v>76683</v>
       </c>
       <c r="V5" s="19">
-        <f>MAX(V6:V36)</f>
+        <f t="shared" si="0"/>
         <v>91181</v>
       </c>
       <c r="W5" s="19">
-        <f>MAX(W6:W36)</f>
+        <f t="shared" si="0"/>
         <v>277830</v>
       </c>
       <c r="X5" s="19">
-        <f>MAX(X6:X36)</f>
+        <f t="shared" si="0"/>
         <v>69313</v>
       </c>
       <c r="Y5" s="9">
-        <f>MAX(Y6:Y36)</f>
+        <f t="shared" si="0"/>
         <v>96.26</v>
       </c>
       <c r="Z5" s="9">
-        <f>MAX(Z6:Z36)</f>
+        <f t="shared" si="0"/>
         <v>299.56</v>
       </c>
       <c r="AA5" s="9">
-        <f>MAX(AA6:AA36)</f>
+        <f t="shared" si="0"/>
         <v>2116.8000000000002</v>
       </c>
       <c r="AB5" s="9">
-        <f>MAX(AB6:AB36)</f>
+        <f t="shared" si="0"/>
         <v>374960</v>
       </c>
       <c r="AC5" s="9">
-        <f>MAX(AC6:AC36)</f>
+        <f t="shared" si="0"/>
         <v>497040</v>
       </c>
       <c r="AD5" s="9">
-        <f>MAX(AD6:AD36)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="AE5" s="9">
-        <f>MAX(AE6:AE36)</f>
+        <f t="shared" si="0"/>
         <v>3320.7</v>
       </c>
       <c r="AF5" s="9">
-        <f>MAX(AF6:AF36)</f>
+        <f t="shared" si="0"/>
         <v>2183.1999999999998</v>
       </c>
     </row>
@@ -21934,15 +21942,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="26585f66-47fc-498d-b213-b46953568bdc">
@@ -21950,6 +21949,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21972,14 +21980,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BCB75A9-047C-49FD-97F3-E954E4582F73}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58DF89A4-C330-4DFA-9A84-C3DE3B38B451}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -21987,4 +21987,12 @@
     <ds:schemaRef ds:uri="26585f66-47fc-498d-b213-b46953568bdc"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BCB75A9-047C-49FD-97F3-E954E4582F73}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated factor names in FinalDataset.xlsx
</commit_message>
<xml_diff>
--- a/FinalDataset.xlsx
+++ b/FinalDataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10727"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rneribar/AIMM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0063FCE4-D74B-7847-AE76-97B309D0608C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2485D8F4-47CD-CF49-BEC3-A1F840291F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="760" windowWidth="29060" windowHeight="17780" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33280" yWindow="1260" windowWidth="29780" windowHeight="26260" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.Original" sheetId="28" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="115">
   <si>
     <t>Year</t>
   </si>
@@ -334,19 +334,58 @@
     <t>TDS (Hueco)</t>
   </si>
   <si>
-    <t>GW TDS (Hueco)</t>
-  </si>
-  <si>
-    <t>SW TDS (Mesilla)</t>
-  </si>
-  <si>
-    <t>SW TDS (Hueco)</t>
-  </si>
-  <si>
     <t>Groundwater  level (Mesilla)</t>
   </si>
   <si>
     <t>Groundwater  level (Hueco)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pecan area </t>
+  </si>
+  <si>
+    <t>Pecan area (MX)</t>
+  </si>
+  <si>
+    <t>Cotton area (MX)</t>
+  </si>
+  <si>
+    <t>Urban area (MX)</t>
+  </si>
+  <si>
+    <t>Alfalfa area (MX)</t>
+  </si>
+  <si>
+    <t>Pecan area (US)</t>
+  </si>
+  <si>
+    <t>Cotton area (US)</t>
+  </si>
+  <si>
+    <t>Urban area (US)</t>
+  </si>
+  <si>
+    <t>Alfalfa area (US)</t>
+  </si>
+  <si>
+    <t>ft below land surface</t>
+  </si>
+  <si>
+    <t>Groundwater quality (Hueco)</t>
+  </si>
+  <si>
+    <t>Surface water supply (EPNo.1)</t>
+  </si>
+  <si>
+    <t>Surface water supply  (EBID)</t>
+  </si>
+  <si>
+    <t>Surface water supply  (Juarez)</t>
+  </si>
+  <si>
+    <t>Surface water quality  (NW El Paso)</t>
+  </si>
+  <si>
+    <t>Surface water quality  (SE El Paso)</t>
   </si>
 </sst>
 </file>
@@ -7757,10 +7796,10 @@
         <v>41</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>42</v>
+        <v>108</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>42</v>
+        <v>108</v>
       </c>
       <c r="AA2" s="9" t="s">
         <v>43</v>
@@ -7781,7 +7820,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:32" s="9" customFormat="1" ht="52" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" s="9" customFormat="1" ht="86" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>47</v>
       </c>
@@ -7819,7 +7858,7 @@
         <v>68</v>
       </c>
       <c r="M3" s="22" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="N3" s="22" t="s">
         <v>13</v>
@@ -7831,55 +7870,55 @@
         <v>15</v>
       </c>
       <c r="Q3" s="22" t="s">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="R3" s="22" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="S3" s="22" t="s">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="T3" s="22" t="s">
-        <v>19</v>
+        <v>103</v>
       </c>
       <c r="U3" s="22" t="s">
-        <v>20</v>
+        <v>104</v>
       </c>
       <c r="V3" s="22" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="W3" s="22" t="s">
-        <v>22</v>
+        <v>106</v>
       </c>
       <c r="X3" s="22" t="s">
-        <v>23</v>
+        <v>107</v>
       </c>
       <c r="Y3" s="22" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="Z3" s="22" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AA3" s="22" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="AB3" s="22" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="AC3" s="22" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="AD3" s="22" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="AE3" s="22" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="AF3" s="22" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:32" ht="205" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" ht="188" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>48</v>
       </c>
@@ -21731,6 +21770,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="26585f66-47fc-498d-b213-b46953568bdc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C0C065D4DE56964884282D8F503EB12D" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cfa0f9876d3650d261453c6251028662">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="26585f66-47fc-498d-b213-b46953568bdc" xmlns:ns3="984dc5cf-9f96-4254-8c6c-2d4fc144aaf2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="61f3943096767e2b3d869813e253bb59" ns2:_="" ns3:_="">
     <xsd:import namespace="26585f66-47fc-498d-b213-b46953568bdc"/>
@@ -21941,16 +21990,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="26585f66-47fc-498d-b213-b46953568bdc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -21961,6 +22000,16 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58DF89A4-C330-4DFA-9A84-C3DE3B38B451}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="26585f66-47fc-498d-b213-b46953568bdc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0E3D96E-C286-4914-9D33-19BF1F42696C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21979,16 +22028,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58DF89A4-C330-4DFA-9A84-C3DE3B38B451}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="26585f66-47fc-498d-b213-b46953568bdc"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BCB75A9-047C-49FD-97F3-E954E4582F73}">
   <ds:schemaRefs>

</xml_diff>